<commit_message>
Econ ledger update 2026-08-23: 6 added, 14 updated, 4 reminder flags
Research pass covering funded Economics Master's/PhD programs:
- Filled placeholder fields on the previously least-detailed/incomplete
  entries (Mannheim CDSE, Hitotsubashi, SNU, HKUST) and refreshed
  urgent/soon/closed programs (ANU, Sydney, Monash, UNSW, Bocconi).
- Added 6 new funded programs: LSE, Warwick, Univ. of Zurich (Zurich
  GSE), Univ. of Copenhagen, Univ. of Hong Kong, and Univ. of Queensland.
- Set 30-day deadline reminder flags on ANU, Monash, Sydney, and the new
  Queensland entry (all have imminent scholarship-round deadlines).
- University of Tokyo (UTIPE) site remains unreachable across two
  research passes — flagged for manual follow-up.
</commit_message>
<xml_diff>
--- a/apps/EconGradAlert/data/tracker.xlsx
+++ b/apps/EconGradAlert/data/tracker.xlsx
@@ -438,7 +438,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last full research pass: 2026-08-22</t>
+          <t>Last full research pass: 2026-08-23</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Program count: 24</t>
+          <t>Program count: 30</t>
         </is>
       </c>
     </row>
@@ -525,12 +525,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y25"/>
+  <dimension ref="A1:Y31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="53" customWidth="1" min="3" max="3"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
@@ -545,13 +545,13 @@
     <col width="60" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="60" customWidth="1" min="17" max="17"/>
-    <col width="32" customWidth="1" min="18" max="18"/>
+    <col width="60" customWidth="1" min="18" max="18"/>
     <col width="60" customWidth="1" min="19" max="19"/>
     <col width="60" customWidth="1" min="20" max="20"/>
     <col width="60" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="14" customWidth="1" min="23" max="23"/>
-    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="60" customWidth="1" min="24" max="24"/>
     <col width="60" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
@@ -730,22 +730,22 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Not published on admissions page</t>
+          <t>7.0 overall minimum (non-native English speakers)</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Not published on admissions page</t>
+          <t>100 iBT minimum</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Not required (not mentioned)</t>
+          <t>Required for applicants without a Dutch degree (Quant score below 160 not competitive); exempt for Dutch-degree holders</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Strong quantitative background; max. 35 students/year; feeds into PhD at UvA/VU/Erasmus</t>
+          <t>Strong quantitative background; max. 35 students/year; feeds into PhD at UvA/VU/Erasmus; 2 academic reference letters</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>1 Dec (scholarship/non-EEA) / 1 Feb (partner non-EEA &amp; EEA scholarship) / 1 May (EEA) — recurring; confirm 2027 dates</t>
+          <t>1 Dec (scholarship/non-EEA) / 1 Feb (partner non-EEA &amp; EEA scholarship) / 1 May (EEA) — recurring; page also notes Cohort 2027-2029 admissions open in Studielink 1 Oct 2026, which is hard to reconcile with the Dec/Feb/May dates shown — cohort-year labeling on the official page is ambiguous, recommend a manual spot-check</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>2 (academic)</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -775,7 +775,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Varies EEA/non-EEA — not published here</t>
+          <t>EEA nationals EUR 2,694 (statutory fee); Non-EEA EUR 20,500 (statutory + institutional fee); no tuition fees during PhD phase</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Scholarships via University of Amsterdam and Tinbergen Institute; apply in December round for best funding chance. Amounts not published.</t>
+          <t>Year 1: full scholarship EUR 1,500/month or partial EUR 750/month. Year 2: full EUR 1,000/month (requires weighted GPA &gt;=8.0 in core courses) or partial EUR 750/month (GPA &gt;=7.5). Institutional fee waivers for selected students (statutory fee not waivable); inter-campus travel compensation also offered.</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -795,17 +795,17 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Filled in IELTS/TOEFL/GRE, references, tuition and scholarship amounts</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; verify deadlines for 2027 cohort</t>
+          <t>Seed entry Aug 2026; deadline year-labeling on official page is internally inconsistent (Dec/Feb/May dates vs. an Oct 2026 Studielink-opening note) — verify manually before relying on exact cohort year</t>
         </is>
       </c>
     </row>
@@ -857,22 +857,22 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Not published on this page</t>
+          <t>7/9 (Academic)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Not published on this page</t>
+          <t>95/120 iBT ("Best Scores")</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Not mentioned on this page</t>
+          <t>Mandatory for all applicants holding a foreign (non-French) degree — Verbal, Quant and Analytical Writing all required; no minimum score published</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>~5 year program; check Admissions section + Student Handbook for full requirements</t>
+          <t>~5 year program; entry is via M2 ETE (doctoral track) then continuation into the PhD — no separate direct-PhD-only application; Cambridge CAE C1 accepted as an alternative to IELTS/TOEFL; exemptions for native English speakers or English-medium degree holders</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -882,27 +882,27 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Not specified on this page — check Admissions section</t>
+          <t>No fixed PhD-only deadline — entry is via the M2 ETE doctoral track. 2026-27 M2 ETE international application window was 10-20 April 2026 (recurring annual spring campaign, ~April) — already closed; next window expected ~April 2027</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>tba</t>
+          <t>later</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>2 minimum, 3 maximum (academic)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
+          <t>None</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
+          <t>International M2 track: EUR 5,500/year + EUR 254 registration fee; fee waivers available on merit/other criteria</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Doctoral school ensures PhD funding; TA/RA positions available. Some M2-level scholarships/grants too.</t>
+          <t>TSE fellowships (EUR 8,000-12,000) allocated to students admitted into the M2 ETE doctoral track; one annual UniCredit Masterscholarship worth EUR 13,000; once in the PhD, "the doctoral school makes sure students receive funding" (mechanism not itemized); TA/RA positions also available at M2 level.</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -922,17 +922,17 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Found entry pathway (via M2 ETE), application window, and language/GRE/fee requirements</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; needs deeper check of Admissions subpage</t>
+          <t>Seed entry Aug 2026; PhD entry is exclusively via the M2 ETE doctoral track, not a standalone PhD application</t>
         </is>
       </c>
     </row>
@@ -1868,57 +1868,57 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>https://www.uni-mannheim.de/gess/apply/admission-requirements/for-cdse/</t>
+          <t>https://www.uni-mannheim.de/gess/programs/cdse/</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Not specified — check admission requirements page</t>
+          <t>No specific score requirement stated on the admission-requirements page</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Not specified — check admission requirements page</t>
+          <t>No specific score requirement stated on the admission-requirements page</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Not specified — check admission requirements page</t>
+          <t>General GRE required, must be taken at an official test center (at-home version not accepted), score no older than 2 years; GRE Subject Test and GMAT not accepted; ETS institution code 0933</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>5-year program (2-yr coursework + 3-yr research); degree awarded: Dr. rer. pol.</t>
+          <t>5-year program (2-yr coursework + 3-yr research); degree awarded: Dr. rer. pol.; letter of motivation (max 500 words, English); transcripts from all institutions attended; Master's in economics or equivalent required (related quantitative fields OK if background sufficient); optional writing sample (English or German); apply only via online portal (gess-application.uni-mannheim.de)</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Not specified — check page</t>
+          <t>Fall intake (exact month/day not specified)</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Not specified — check admission requirements page</t>
+          <t>31 March annually (final deadline for Fall intake, recurring); applications open ~mid-November prior year; early-admission deadline ~15 January</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>tba</t>
+          <t>later</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>2 (from faculty)</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not found — likely none (consistent with typical German public-university no-fee doctoral admission), unconfirmed</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not found — likely none (German public university), unconfirmed</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1928,7 +1928,7 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>CDSE commits to funding students for the full program duration, contingent on successful completion of the course phase and academic standing.</t>
+          <t>CDSE commits to funding students for the full 5-year program duration, contingent on successful completion of the course phase and academic standing — typically scholarship in years 1-2, then research-assistant positions afterward. ZEW Cooperation Track additionally offers EUR 1,500/month in the first year for students who opt in.</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
@@ -1938,17 +1938,17 @@
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Filled in deadline, GRE/reference requirements, and ZEW Cooperation Track funding detail — previously the least-detailed entry</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; least-detailed entry so far, prioritise for next refresh</t>
+          <t>Seed entry Aug 2026; application/tuition fees still unconfirmed</t>
         </is>
       </c>
     </row>
@@ -2000,22 +2000,22 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>No numeric threshold; general requirement is B2 (CEFR) English, via valid IELTS/TOEFL score or self-declaration for native speakers/English-taught degree holders</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>See IELTS field — B2 (CEFR) equivalent required, no specific numeric score published</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>GRE or GMAT required for most PhD programs (PhD in Legal Studies is the stated exception); Bocconi GRE recipient code 1517</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>42nd cycle referenced for 2026-27; check 'Preparing to Apply' subpage for full requirements</t>
+          <t>42nd cycle referenced for 2026-27; statement of purpose (max 1,200 words) describing motivation, research interests and goals</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -2025,27 +2025,27 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Ordinary cycle ~October (closed); special FIS-funded call ~18 May 2026 — confirm annual pattern</t>
+          <t>Both the 42nd-cycle (2026-27) ordinary call and the special FIS-funded call (deadline was 18 May 2026) have now closed; the 43rd cycle (2027-28) has not yet been announced as of 23 Aug 2026 — recurring annual pattern (ordinary call ~October, FIS-funded call ~spring), check back autumn/winter 2026</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>soon</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Up to 2</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Free — no application fee</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not confirmed — PhD is generally funded/no tuition for admitted students, but no explicit figure located</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>Standard funded positions in ordinary admissions cycle, plus a dedicated FIS (Fondo Italiano per la Scienza) funded call seen for 2026.</t>
+          <t>Standard funded positions in ordinary admissions cycle, plus a dedicated FIS (Fondo Italiano per la Scienza) funded call seen for 2026 (amount/coverage not confirmed this pass — FIS call page unreachable).</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
@@ -2065,17 +2065,17 @@
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Confirmed 2026-27 cycle (ordinary + FIS call) is fully closed and 2027-28 cycle not yet announced; added test-requirement and application-fee detail</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026</t>
+          <t>Seed entry Aug 2026; watch for 43rd-cycle (2027-28) announcement in autumn/winter 2026</t>
         </is>
       </c>
     </row>
@@ -2209,77 +2209,77 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>EUR-13</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>MRes/PhD</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>MRes/PhD in Economics</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>National University of Singapore (NUS)</t>
+          <t>London School of Economics (LSE)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>#120</t>
+          <t>#16</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>London</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://fass.nus.edu.sg/ecs/doctor-of-philosophy-economics/</t>
+          <t>https://www.lse.ac.uk/study-at-lse/graduate/mresphd-economics</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Not mentioned (standard faculty requirement applies)</t>
+          <t>Not specified on this page (English test required 'if applicable'; no threshold published there)</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Not mentioned (standard faculty requirement applies)</t>
+          <t>Not specified on this page</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Not mentioned on this page</t>
+          <t>Required for all applicants (score must be &lt;5 years old); most successful applicants score ~166+ Quant</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Non-English-medium graduates may need to take a Graduate English Course</t>
+          <t>Research statement (5 prompts, ~200 words each), statement of academic purpose (~1,000 words), CV, transcripts</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>August 2026 (intro Maths/Stats course), full program starts thereafter</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Early: 30 September 2026; Main: 1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
+          <t>10 December (recurring annual; most recent was 10 Dec 2025 for 2026 entry, next expected ~Dec 2026)</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -2289,261 +2289,261 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>2 (academic)</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
+          <t>Not specified (fee mentioned but amount not published on this page)</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Not detailed (fully funded — see funding)</t>
+          <t>2026/27 rates: Home GBP 5,238/yr; Overseas GBP 24,400/yr (waived for funded students)</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Yes — all admitted students</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>Full financial support (fees + living expenses) for 5 years: NUS Research Scholarship (years 1-4), department funding (year 5), plus research/travel allowance.</t>
+          <t>LSE PhD Studentships and ESRC studentships cover fees + stipend for eligible admits; department also offers scholarship packages plus paid TA/RA work after year 1; funding deadline is same as application deadline.</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; contact econ-phd@nus.edu.sg for specifics</t>
+          <t>One of the top-ranked UK econ PhDs; verify current-cycle deadline/fee figures directly on LSE site before applying, as dates shift annually.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>EUR-14</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MPhil/PhD</t>
+          <t>MRes/PhD</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics</t>
+          <t>MRes/PhD in Finance &amp; Economics</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Hong Kong University of Science and Technology (HKUST)</t>
+          <t>University of Warwick (Warwick Business School)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>#287</t>
+          <t>#37</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Hong Kong (China)</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Coventry</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://econ.hkust.edu.hk/programs-n-courses/mphd/mphd-admission</t>
+          <t>https://www.wbs.ac.uk/courses/doctoral/mres-phd-finance-economics/how-to-apply/</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>Not specified on program page (English test certificate required, threshold not published there)</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Required if non-English-medium background (score not published here)</t>
+          <t>Not specified on program page</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Required ("satisfactory score")</t>
+          <t>GRE or GMAT score required (no minimum published)</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Conditional offers require official documents by end of July</t>
+          <t>Personal statement, CV, transcripts/certificates; 2 academic references must arrive by the deadline or the application is rejected</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Fall semester</t>
+          <t>Late September (next start likely Sept 2027, recurring)</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
+          <t>31 January (recurring annual; most recently 31 Jan 2026 for Sept 2026 entry)</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>soon</t>
+          <t>later</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
+          <t>2 (academic)</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>Not disclosed</t>
-        </is>
-      </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Program described as fully-funded for both Home and International students (fees covered as part of funding package)</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>Likely (via HKPFS / dept funding — see ASA-03)</t>
+          <t>Yes — all successful applicants</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>Not detailed on this page directly — cross-reference Hong Kong PhD Fellowship Scheme (ASA-03) and department stipends.</t>
+          <t>All successful applicants receive full fee waiver + stipend + a research/conference travel budget; exact stipend amount not published on this page (contact PhdAdmissions@wbs.ac.uk for figure). Warwick Doctoral College also runs a separate scholarship competition (deadline ~11 Dec) that WBS students are automatically considered for.</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026</t>
+          <t>Competitive, limited places on the Doctoral College scholarship track; confirm stipend amount directly with admissions.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ASA-03</t>
+          <t>EUR-15</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PhD (Fellowship, cross-university)</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Hong Kong PhD Fellowship Scheme (HKPFS)</t>
+          <t>PhD in Economics (Zurich Graduate School of Economics)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
+          <t>University of Zurich</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Varies by host university (scheme spans multiple HK institutions)</t>
+          <t>#32</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Hong Kong (China)</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>https://www.gs.cuhk.edu.hk/admissions/scholarships-fees/hkpfs</t>
+          <t>https://www.econ.uzh.ch/en/study/phd/zurichgse/howtoapply.html</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules (set by individual dept/program)</t>
+          <t>Accepted for non-Bologna-country applicants without English-language prior education (specific band not published)</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules (set by individual dept/program)</t>
+          <t>Accepted alternative to IELTS; CPE/CAE also accepted</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules (set by individual dept/program)</t>
+          <t>Strongly recommended for all; mandatory for applicants with degrees from non-Bologna (non-European) countries</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Apply via 2 parallel channels: RGC website (choose up to 2 programmes) AND university's own online system, quoting HKPFS reference number. Selection on academic excellence, research potential, communication, leadership.</t>
+          <t>Compulsory pre-sessional Introductory Maths course (mid-August, before Fall term); Track B (after Master's) or Track C 'Fast Track' (after strong Bachelor's)</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Typically September (Fall)</t>
+          <t>Fall term (~September)</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>1 December 2026, 12:00 noon HKT (RGC) / 11:59pm HKT (university, e.g. CUHK)</t>
+          <t>15 January annually (applications open each October)</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>soon</t>
+          <t>later</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -2553,44 +2553,44 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>Waived (see funding)</t>
+          <t>Not specified (Swiss public universities have low nominal tuition, typically a few hundred CHF/semester)</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Yes — major fellowship</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>~HK$1.81 million total (~US$232,400): stipend HK$344,400/yr (~US$44,200), conference/travel HK$14,400/yr, tuition waiver up to HK$198,000, lodging award up to HK$100,000, first-year hostel waiver.</t>
+          <t>Most candidates receive departmental scholarships from the first year; additional funding via URPP and the UBS Center Scholarship (a competitive full annual scholarship worth ~CHF 42,500/year) available to advanced students later in the program.</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; this is a cross-institution scheme, not a single program — apply through chosen university's Economics dept</t>
+          <t>Highly selective — ~400 applications/year for only ~12-15 admits; confirm current-year scholarship amount directly with the department.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ASA-04</t>
+          <t>EUR-16</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2600,72 +2600,72 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>PhD Programme in Economics</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Nanyang Technological University (NTU Singapore)</t>
+          <t>University of Copenhagen (Department of Economics)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>#253</t>
+          <t>#54</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Copenhagen</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>https://www.ntu.edu.sg/education/graduate-programme/ph.d.-in-economics</t>
+          <t>https://www.economics.ku.dk/phd/til-ansoegere/</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>7.0 minimum (preferred)</t>
+          <t>Not specified on department page</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>105 minimum</t>
+          <t>Not specified on department page</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Not mandatory, but scores considered if submitted; recommended for non-Singapore-university degree holders</t>
+          <t>Not mentioned as a requirement</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Scores must be within 2 years of application; exemptions for native speakers / English-medium degree holders</t>
+          <t>Must have completed coursework in Macro, Micro, and Econometrics; must contact a prospective supervisor before applying; non-English/Scandinavian degree holders need certified translations of transcripts</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>New PhD students typically start in the fall; vacant scholarships announced once a year</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Not specified on this page — contact ac-sss-ge@ntu.edu.sg</t>
+          <t>15 January (recurring annual round; individual scholarship postings can have their own deadlines, some closing May/June)</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>tba</t>
+          <t>later</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -2680,44 +2680,44 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>Not specified (MOE-subsidised place)</t>
+          <t>Funded/scholarship track: salaried position, no fee; self-funded (non-scholarship) track reported at DKK 50,000/year — verify before relying on this figure</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes — salaried position</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>MOE-subsidised programme; Nanyang Research Scholarship available for qualifying students.</t>
+          <t>PhD scholarship holders are university employees on the Danish state academic-union pay scale — basic salary ~DKK 29,700/month plus a ~DKK 1,550/month PhD supplement (roughly EUR 4,150/month total, 2025 rates); Danmarks Nationalbank also offers external fellowships for macro/finance-focused PhD students.</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; deadline needs manual confirmation</t>
+          <t>Danish PhDs are structured as paid jobs rather than stipends, so funding is unusually generous and reliable versus many EU peers; no published IELTS/TOEFL threshold found — confirm with department.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2727,17 +2727,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD)</t>
+          <t>PhD in Economics</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>University of Tokyo</t>
+          <t>National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>#110</t>
+          <t>#120</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2747,77 +2747,77 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Tokyo</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>https://www.gaia.e.u-tokyo.ac.jp/utipe/</t>
+          <t>https://fass.nus.edu.sg/ecs/doctor-of-philosophy-economics/</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not mentioned (standard faculty requirement applies)</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not mentioned (standard faculty requirement applies)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not mentioned on this page</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>English-taught international program; site access was unreliable during this research pass</t>
+          <t>Non-English-medium graduates may need to take a Graduate English Course; good undergraduate honours degree (first class or high 2:1 equivalent) or Master's, in economics or another quantitative subject</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not specified on this page</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Not yet confirmed — needs manual check</t>
+          <t>Early: 30 September 2026; Main: 1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>tba</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not detailed (fully funded — see funding)</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Likely (MEXT scholarship-eligible — common for UTokyo international programs)</t>
+          <t>Yes — all admitted students</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>Not confirmed this pass — MEXT (Japanese government) scholarship route is commonly available for this program; needs verification.</t>
+          <t>Full financial support (fees + living expenses) for 5 years: NUS Research Scholarship (years 1-4), department funding (year 5), plus research/travel allowance.</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
@@ -2827,44 +2827,44 @@
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Confirmed deadlines unchanged; added admission requirement detail</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>INCOMPLETE — prioritise for next weekly refresh; fetch blocked this pass</t>
+          <t>Seed entry Aug 2026; contact econ-phd@nus.edu.sg for specifics</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>ASA-02</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>MPhil/PhD</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD)</t>
+          <t>MPhil/PhD in Economics</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Hitotsubashi University</t>
+          <t>Hong Kong University of Science and Technology (HKUST)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Not in top 300</t>
+          <t>#287</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2874,77 +2874,77 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Hong Kong (China)</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Tokyo (Kunitachi)</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>https://www.hit-u.ac.jp/eng/admissions/</t>
+          <t>https://econ.hkust.edu.hk/programs-n-courses/mphd/mphd-admission</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>6.5 overall, no subscore below 5.5 (university-wide standard; waived if English-medium/first-language English)</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>iBT 80 / pBT 550 / Revised PBT 60 (university-wide standard)</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Required ("satisfactory score")</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Known for strong English-taught economics research programs</t>
+          <t>Conditional offers require official documents by end of July</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Fall semester</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Not yet confirmed — needs manual check</t>
+          <t>1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>tba</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>HK$180, non-refundable</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>HK$47,000/year (2026/27 rate, full-time or part-time)</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>Likely (MEXT scholarship-eligible)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>Not confirmed this pass — needs verification against department page.</t>
+          <t>Postgraduate Studentship (PGS): HK$229,620/year (2025/26 rate); recipients serve as Graduate Teaching Assistants. HKUST RedBird PhD Award stacks with HKPFS: Recruitment Award HK$40,000 (year 1) + Academic Excellence Award HK$20,000/year (later years). Conference &amp; Travel Allowance ~HK$14,200/year for HKPFS holders. Also cross-reference Hong Kong PhD Fellowship Scheme (ASA-03).</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
@@ -2954,44 +2954,44 @@
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr), fees, and IELTS/TOEFL standards; upgraded funding_status from Likely to Yes</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>INCOMPLETE — prioritise for next weekly refresh</t>
+          <t>Seed entry Aug 2026</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>ASA-03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>PhD (Fellowship, cross-university)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD)</t>
+          <t>Hong Kong PhD Fellowship Scheme (HKPFS)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Seoul National University (SNU)</t>
+          <t>Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>#189</t>
+          <t>Varies by host university (scheme spans multiple HK institutions)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -3001,77 +3001,77 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Hong Kong (China)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Seoul</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>https://en.snu.ac.kr/admission</t>
+          <t>https://www.gs.cuhk.edu.hk/admissions/scholarships-fees/hkpfs</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Not yet confirmed at dept level</t>
+          <t>Not specified in scheme rules (set by individual dept/program)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Not yet confirmed at dept level</t>
+          <t>Not specified in scheme rules (set by individual dept/program)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Not yet confirmed at dept level</t>
+          <t>Not specified in scheme rules (set by individual dept/program)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>University-wide scholarships identified; department-level participation not yet confirmed</t>
+          <t>Apply via 2 parallel channels: RGC website (choose up to 2 programmes) AND university's own online system, quoting HKPFS reference number. Selection on academic excellence, research potential, communication, leadership.</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Typically September (Fall)</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Not yet confirmed at dept level — scholarship deadlines below are university-wide</t>
+          <t>1 December 2026, 12:00 noon HKT (RGC) / 11:59pm HKT (university, e.g. CUHK)</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>tba</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not specified in scheme rules</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Waived (see funding)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>Likely (university-wide scholarships)</t>
+          <t>Yes — major fellowship</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>Global Korea Scholarship: full tuition (6 semesters) + ~1.4M KRW/month + airfare (Korean language req., TOPIK 3; deadline ~February). SNU President Fellowship: full tuition + 1.5-2M KRW/month. Grad Scholarship for Excellent Foreign Students: full tuition (4 semesters) + 500K KRW/month min. Dept-level applicability not yet confirmed.</t>
+          <t>~HK$1.81 million total (~US$232,400): stipend HK$344,400/yr (~US$44,200), conference/travel HK$14,400/yr, tuition waiver up to HK$198,000, lodging award up to HK$100,000, first-year hostel waiver.</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
@@ -3091,14 +3091,14 @@
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>INCOMPLETE — prioritise for next weekly refresh</t>
+          <t>Seed entry Aug 2026; this is a cross-institution scheme, not a single program — apply through chosen university's Economics dept</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-04</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3113,72 +3113,72 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Australian National University (ANU)</t>
+          <t>Nanyang Technological University (NTU Singapore)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>#124</t>
+          <t>#253</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Canberra</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>https://cbe.anu.edu.au/study/graduate-research-programs/doctor-philosophy-phd/phd-economics</t>
+          <t>https://www.ntu.edu.sg/education/graduate-programme/ph.d.-in-economics</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>6.5 overall (no band below 6.0)</t>
+          <t>7.0 minimum (preferred)</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>570 (paper-based; essay ≥4.5)</t>
+          <t>105 minimum</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Mandatory (code 7833); exempt if ANU Econ Honours/Masters</t>
+          <t>Not mandatory, but scores considered if submitted; recommended for non-Singapore-university degree holders</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Pre-PhD summer course required, Jan-Feb, arriving 4-6 weeks before semester</t>
+          <t>Scores must be within 2 years of application; exemptions for native speakers / English-medium degree holders</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>February (Semester 1); Semester 2 entry possible (July)</t>
+          <t>Not specified on this page</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>For Feb 2027 start: international scholarship applicants before 31 Aug 2026 (imminent), standard before 31 Oct 2026; Sem 2 entry before 31 Mar</t>
+          <t>Not specified on this page — contact ac-sss-ge@ntu.edu.sg</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>urgent</t>
+          <t>tba</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -3188,7 +3188,7 @@
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not specified (MOE-subsidised place)</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>HDR scholarships available — see CBE 'Scholarships and Fees' page for amounts.</t>
+          <t>MOE-subsidised programme; Nanyang Research Scholarship available for qualifying students.</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
@@ -3218,14 +3218,14 @@
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026 — international scholarship deadline is very close, verify immediately on the program page</t>
+          <t>Seed entry Aug 2026; deadline needs manual confirmation</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3235,67 +3235,67 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics</t>
+          <t>International Program in Economics (PhD)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>University of Melbourne</t>
+          <t>University of Tokyo</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>#151</t>
+          <t>#110</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Melbourne</t>
+          <t>Tokyo</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>https://study.unimelb.edu.au/find/courses/graduate/doctoral-program-in-economics/how-to-apply/</t>
+          <t>https://www.gaia.e.u-tokyo.ac.jp/utipe/</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>7.0 overall (7.0 writing, no band below 6.0)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>94 iBT (W27/S18/R13/L13)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Not mentioned in entry requirements</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>PTE Academic 72+ (written 75+); CAE 185+ also accepted; 5-year program (2 coursework + 3 research)</t>
+          <t>English-taught international program; site (gaia.e.u-tokyo.ac.jp) unreachable again this pass — DNS resolution failure confirmed via two independent fetch methods, same issue as prior pass</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>March intake</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Not specified on this page — check application key dates page</t>
+          <t>Not yet confirmed — needs manual check</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -3305,27 +3305,27 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>Not detailed (RTP places available)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Likely (MEXT scholarship-eligible — common for UTokyo international programs)</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>Australian Government Research Training Program (RTP) funded places available.</t>
+          <t>Not confirmed this pass — MEXT (Japanese government) scholarship route is commonly available for this program; needs verification.</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
@@ -3335,24 +3335,24 @@
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Site unreachable again (DNS failure) — no field data updated; flagged an unconfirmed lead on a possible admission-policy change</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026</t>
+          <t>INCOMPLETE — prioritise for next refresh. Unconfirmed search snippets suggest UTIPE's PhD admission policy changed circa 2023 to require completing UTIPE's own Master's program first (may no longer accept direct external PhD applicants) — not verified against the primary source, needs a manual check.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3362,67 +3362,67 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>PhD (Economics)</t>
+          <t>Graduate School of Economics (PhD)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Monash Business School</t>
+          <t>Hitotsubashi University</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>#46</t>
+          <t>#390 (confirmed still outside global top 300)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Melbourne (Clayton)</t>
+          <t>Tokyo (Kunitachi)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>https://www.monash.edu/business/research/phd-programs/scholarships-and-fees</t>
+          <t>https://www.econ.hit-u.ac.jp/eng/page/graduate/admission.html</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>Not stated (page mentions TOEFL/TOEIC only)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>TOEFL or TOEIC score required as part of application materials; specific minimum score not stated</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Multiple named scholarships stack with base RTP/Monash funding</t>
+          <t>Two intakes/year (Spring and Autumn); international applicants without a Hitotsubashi Master's apply via an AO exam route — either general AO (2+ years work experience post-master's) or AO for international applicants with a Master's from outside Japan; admission mainly via submitted documents, interview may follow (online option for overseas applicants)</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>Spring or Autumn intake (two cycles/year)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>Applications open ~October (for the following Spring start) and ~April (for the following Autumn start); exact day-level deadlines are issued per-cycle in a separate department announcement, not found this pass</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -3432,27 +3432,27 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>At least 1 recommendation letter required (exact number not specified)</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Likely (MEXT scholarship-eligible)</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>Donald Cochrane Scholarship: AUD 10,000/yr x 3.5yrs (3 awarded/yr). Dean's Excellence Award: up to AUD 5,000/yr top-up (10/yr). Graduate Research Scholarship: AUD 41,000/yr tuition (~12/yr). Plus university-wide Monash Graduate Scholarship / RTP places.</t>
+          <t>MEXT scholarship route confirmed to exist, administered via a separate central international-office page (requires embassy/consulate preliminary candidacy). No department-specific stipend/assistantship figures found.</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
@@ -3462,24 +3462,24 @@
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Located the correct department admissions page (previous link was a generic university page); found intake-cycle pattern, AO exam routes, and precise RePEc rank (#390)</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026</t>
+          <t>Partially complete — exact per-cycle deadline dates and funding figures still needed; prioritise for next refresh</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3489,97 +3489,97 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>Department of Economics (PhD)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>University of Sydney</t>
+          <t>Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>#87</t>
+          <t>#189</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Sydney</t>
+          <t>Seoul</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>https://www.sydney.edu.au/scholarships/</t>
+          <t>https://en.snu.ac.kr/admission</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Not specified at general program level</t>
+          <t>6.0 minimum (university-wide standard)</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Not specified at general program level</t>
+          <t>iBT 80, or TEPS 551 (university-wide standard, alternative to IELTS)</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
+          <t>Not required (no GRE requirement found in central admissions materials)</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Example named scholarship seen (topic-restricted, econ conflict/ag markets) — general program funding likely via RTP</t>
+          <t>University-wide scholarships identified; department-level participation not yet confirmed</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Varies by scholarship round — check scholarships portal</t>
+          <t>University-wide pattern: Fall-intake applications open ~early March (2026 Fall: 3-5 Mar); Spring-intake applications open ~early July (2027 Spring: 6-9 Jul) — both 2026 cycles already closed; 2027 Fall cycle not yet announced. Department-specific PhD deadline still not separately confirmed.</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>tba</t>
+          <t>later</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>1 (for named scholarship example; general program may differ)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>KRW 90,000 (no fee waivers offered)</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Likely (university-wide scholarships)</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>RTP-style stipend scholarships ~AUD 41,753/yr (base AUD 37,207 + top-up), up to 3 years, seen via School of Economics named scholarship. General RTP funding also available for the PhD program broadly.</t>
+          <t>Global Korea Scholarship: full tuition (6 semesters) + ~1.4M KRW/month + airfare (Korean language req., TOPIK 3; deadline ~February). SNU President Fellowship: full tuition + 1.5-2M KRW/month. Grad Scholarship for Excellent Foreign Students: full tuition (4 semesters) + 500K KRW/month min. Dept-level applicability not yet confirmed — search turned up only informal/unofficial claims (e.g. individual professors self-funding RAs from grants), not an official department statement.</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
@@ -3589,144 +3589,906 @@
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Found university-wide test-score/fee requirements and admission-cycle pattern; department-specific PhD funding still unconfirmed</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; needs a general (non-topic-restricted) funding page check</t>
+          <t>Department-level Economics PhD funding not yet confirmed — university-wide scholarships only; prioritise for next refresh</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>ASA-08</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>PhD</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>PhD in Business (Economics track)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>University of Hong Kong (Faculty of Business and Economics)</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>#106</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Hong Kong (China)</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Hong Kong</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>https://phd.hkubs.hku.hk/admissions/admission-application-and-tuition-fee</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Academic overall 6.5, all subtests &gt;= 6.0 (waived if prior degree was taught in English)</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>iBT &gt;= 85</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>GRE or GMAT required, score &lt;5 years old (institution codes: GRE 2482, GMAT FS2-WL-48)</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Bachelor's with first-class honours (or equivalent), or Bachelor's + Master's from a recognized university; 3-year track with a research Master's, 4-year track without one; Economics is one of six FBE PhD fields</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Fall semester, normally September (matriculates once a year)</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Applications open 1 September; Main Round closes 1 December (recurring annual cycle; late applications considered only if places remain)</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>soon</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>2 (academic referee reports, submitted directly by referees)</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>HK$600 (paid online via HKU Graduate School application system)</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>HK$49,500/year (2027-28 rate) for full-time PhD — typically waived/covered for scholarship holders</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>Standard Postgraduate Scholarship (PGS) pays HK$19,135/month (rising to HK$19,655/month once candidature is confirmed), available to essentially all admitted PhD students regardless of HKPFS status. HKPFS awardees instead receive HK$28,700/month plus HK$14,400/year travel allowance for up to 3 years.</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>Added (new find)</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>Distinct from the cross-institution HKPFS scheme already tracked (ASA-03) — nearly all admitted PhD students get baseline PGS funding here even without winning HKPFS, a broader guarantee than HKPFS alone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>AUS-01</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>PhD</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>PhD in Economics</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Australian National University (ANU)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>#124</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Canberra</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>https://cbe.anu.edu.au/study/graduate-research-programs/doctor-philosophy-phd/phd-economics</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>6.5 overall (no band below 6.0)</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>570 (paper-based; essay ≥4.5)</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Mandatory (code 7833); exempt if ANU Econ Honours/Masters</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Pre-PhD summer course required, Jan-Feb, arriving 4-6 weeks before semester</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>February (Semester 1); Semester 2 entry possible (July)</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>For Feb 2027 start: international scholarship applicants before 31 Aug 2026 (imminent), standard before 31 Oct 2026; Sem 2 entry before 31 Mar</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>urgent</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>Australian Government RTP Stipend: AUD $39,069/year (2026 full-time base rate, ANU-wide), paid fortnightly, up to 3.5 years. Some HDR supplementary scholarships add AUD $7,000/year on top, for up to 3 years. Domestic candidates pay no tuition (RTP-covered); international candidates can compete for HDR Fee Remission Merit Scholarships covering up to 4 years.</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>Confirmed the 31 Aug 2026 international scholarship deadline is still live (verified directly on program page); added RTP stipend figures; set 30-day reminder flag</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>Seed entry Aug 2026 — international scholarship deadline is imminent (8 days away as of this update)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>AUS-02</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>PhD</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Doctoral Program in Economics</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>University of Melbourne</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>#151</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>https://study.unimelb.edu.au/find/courses/graduate/doctoral-program-in-economics/how-to-apply/</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>7.0 overall (7.0 writing, no band below 6.0)</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>94 iBT (W27/S18/R13/L13)</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Not mentioned in entry requirements</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>PTE Academic 72+ (written 75+); CAE 185+ also accepted; 5-year program (2 coursework + 3 research)</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>March intake</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>March 2027 intake deadline reported as 30 November 2026 — found via search summary only; the official how-to-apply/key-dates pages returned HTTP 403 on every direct fetch attempt this pass, so this date is unconfirmed by primary source and should be manually verified</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>soon</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Not mentioned</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>Not detailed — full tuition fee waiver reported (see funding)</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>Australian Government Research Training Program (RTP) funded places available: RTP stipend reported at AUD $39,500/year (2026 rate) plus full tuition fee waiver and AUD $15,000 research/conference travel funding for confirmed PhD candidates (unconfirmed by primary source — see deadline note). Program structure: 2-year Master of Commerce coursework + 3-year PhD.</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>Found a reported deadline and funding figures via search, but could not confirm via direct page fetch (403 blocked) — flagged as lower confidence</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>Seed entry Aug 2026; unimelb.edu.au pages returned HTTP 403 to automated fetches this pass — recommend a manual browser check before relying on the reported 30 Nov 2026 deadline</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>AUS-03</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>PhD</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>PhD (Economics)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Monash Business School</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>#46</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Melbourne (Clayton)</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>https://www.monash.edu/business/research/phd-programs/scholarships-and-fees</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>7.0 minimum reported (third-party source, not confirmed on official Monash page — page returned HTTP 403 to direct fetch)</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>94 minimum reported (same caveat as IELTS — unconfirmed by primary source)</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Not specified on this page</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Multiple named scholarships stack with base RTP/Monash funding</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Not specified on this page</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Two pathways found (via search — official pages returned HTTP 403 to direct fetch, unconfirmed by primary source): Integrated PhD program (Master of Commerce + PhD), Feb/Semester-1 entry — applications open 1 Jul-31 Aug (closing imminently); Jul/Semester-2 entry — applications open 1 Dec-1 Feb. Separately, general Graduate Research Scholarship rounds: international Round 1 closes 31 Mar, Round 3 closes ~31 Jul/31 Aug; domestic Round 2 closes 31 May, Round 4 closes 31 Oct.</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>urgent</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>International ~AUD $38,900/yr, domestic ~AUD $37,100/yr reported (third-party aggregator source, not confirmed by official Monash page)</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>Donald Cochrane Scholarship: AUD 10,000/yr x 3.5yrs (3 awarded/yr). Dean's Excellence Award: up to AUD 5,000/yr top-up (10/yr). Graduate Research Scholarship: AUD 41,000/yr tuition (~12/yr). Plus university-wide Monash Graduate Scholarship / RTP places.</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>Found application-window pattern suggesting an imminent (~31 Aug) integrated-pathway deadline, plus fee/test figures — all via search snippets/third-party sites since monash.edu returned HTTP 403 on every direct fetch attempt; set 30-day reminder flag pending confirmation</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>Seed entry Aug 2026; monash.edu blocked all automated fetches this pass (scholarships-and-fees, apply, and program pages all 403'd) — every figure in this update is lower-confidence (search snippets/third-party aggregator only) and needs a manual browser check, especially the reported 31 Aug 2026 integrated-pathway deadline</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>AUS-04</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>PhD</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>PhD in Economics</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>University of Sydney</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>#87</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>https://www.sydney.edu.au/scholarships/</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Not specified at general program level</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Not specified at general program level</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Not mentioned</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Example named scholarship seen (topic-restricted, econ conflict/ag markets) — general program funding likely via RTP. Material finding: Sydney has no dedicated 'PhD in Economics' program page — the Economics coursework handbook explicitly states it "does not include a research component and thus does not provide a pathway to higher degree by research (e.g. PhD) studies." PhD study is pursued via the general Doctor of Philosophy degree with a nominated Economics supervisor/discipline, not a single named landing page.</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Not specified on this page</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>General Research Training Program (RTP) scholarship rounds for 2027 entry (found via search, not a directly-fetched dedicated Economics PhD page): Research Period 1 &amp; 2 — deadline 11 September 2026; Research Period 3 &amp; 4 — deadline 18 December 2026.</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>urgent</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>1 (for named scholarship example; general program may differ)</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>RTP-style stipend scholarships ~AUD 41,753/yr (base AUD 37,207 + top-up), up to 3 years, seen via School of Economics named scholarship. General RTP funding also available for the PhD program broadly.</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>Found general RTP scholarship round deadlines (11 Sep / 18 Dec 2026); confirmed there is no dedicated Sydney 'PhD in Economics' page — entry is via the general PhD degree with an Economics supervisor; set 30-day reminder flag</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>Seed entry Aug 2026; needs a general (non-topic-restricted) funding page check; no dedicated Economics-specific PhD admissions page exists at Sydney</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>AUS-05</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>PhD in Economics</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>UNSW Sydney</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>#80</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>Sydney</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>https://www.unsw.edu.au/business/study-with-us/postgraduate-research/phd-degrees/doctor-philosophy-phd-economics</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>Not listed on this page (exemptions for English-speaking-country citizens)</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>Not listed on this page</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>Optional but recommended</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>Alternative English tests: PTE, Cambridge, or UNSW Global English Course</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Not listed on this page (exemptions for AU/CA/UK/US/NZ citizens); non-English-speaking-country applicants need IELTS/TOEFL/PTE/Cambridge or the UNSW Global English Course</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Not listed on this page — see IELTS field for alternatives</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Optional but recommended overall; one source indicates GRE may be specifically required for the Economics stream — this conflicts with the general 'optional' language elsewhere and needs manual confirmation</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Alternative English tests: PTE, Cambridge, or UNSW Global English Course. Program begins with a 1-year Master of Pre-Doctoral Business Studies, followed by 3-3.5 years of doctoral research; direct entry to the 3-year PhD is possible for candidates with first-class Honours/Master's plus independent funding (Stream 2).</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
         <is>
           <t>Term 1 – February</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>Most recent Expression of Interest window closed 15 August 2026 (one week before this tracker's research date) — next EOI window not yet announced, check page</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Confirmed still closed as of 23 Aug 2026 (verified directly on program page): EOI window opened 20 March 2026, closed 15 August 2026, no newer/next EOI window posted. Note: a separate 26 August 2026 formal-application deadline exists, but it applies only to candidates already invited to apply from the closed EOI round, not to new applicants.</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
         <is>
           <t>closed</t>
         </is>
       </c>
-      <c r="Q25" t="inlineStr">
+      <c r="Q30" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="R25" t="inlineStr">
+      <c r="R30" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="S25" t="inlineStr">
+      <c r="S30" t="inlineStr">
         <is>
           <t>Not detailed (fully funded — see funding)</t>
         </is>
       </c>
-      <c r="T25" t="inlineStr">
+      <c r="T30" t="inlineStr">
         <is>
           <t>Yes — all admitted students</t>
         </is>
       </c>
-      <c r="U25" t="inlineStr">
+      <c r="U30" t="inlineStr">
         <is>
           <t>Full tuition waiver + stipend AUD 35,000-45,000/yr, up to 4.5 years (+1 optional fellowship year), plus substantial research/conference travel funding.</t>
         </is>
       </c>
-      <c r="V25" t="inlineStr">
+      <c r="V30" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="W25" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
-      <c r="X25" t="inlineStr">
-        <is>
-          <t>Added (seed)</t>
-        </is>
-      </c>
-      <c r="Y25" t="inlineStr">
-        <is>
-          <t>Seed entry Aug 2026 — EOI window just closed, watch for the next one to open</t>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>Confirmed EOI window remains closed with no new window announced; added program structure and English-test details</t>
+        </is>
+      </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>Seed entry Aug 2026 — EOI window closed 15 Aug 2026, still no next window announced as of this update</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>AUS-06</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>PhD</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Doctor of Philosophy (Economics)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>University of Queensland (School of Economics)</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>#71</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Brisbane</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>https://economics.uq.edu.au/study/phd</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Academic overall 6.5, with 6.0 minimum in each of reading/writing/speaking/listening</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Not specified on the economics-specific page (UQ university-wide PhD pages generally accept TOEFL iBT as an alternative to IELTS)</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Not confirmed as required; application package can include GRE/GMAT score sheets, suggesting optional/supplementary rather than mandatory</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Academic CV, transcripts; MPhil/research master's options also available; can join a funded project with scholarship support as an alternative entry route</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Quarterly intakes (research quarters begin 1 Jan, 1 Apr, 1 Jul, 1 Oct); applications for RHD programs can be submitted any time</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Rolling application, but scholarship rounds close on fixed dates — 31 August 2026 and 19 October 2026 rounds cited for upcoming 2027 research quarters</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>urgent</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>Minimum 2 referee reports</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>Not specified (international RTP scholarship recipients typically get a full tuition fee offset)</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>RTP/UQGRSS provides a tax-free living stipend of AUD $37,500/year (2026 rate, indexed annually) plus, for eligible international candidates, a tuition fee offset; no separate application needed beyond the program EOI.</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>Added (new find)</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>Scholarship is university-wide (RTP/UQGRSS), not economics-specific, but School of Economics PhD candidates are eligible; confirm current-cycle scholarship closing dates on the UQ Scholarships portal since they shift each year. The 31 Aug 2026 round is imminent.</t>
         </is>
       </c>
     </row>
@@ -3741,14 +4503,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="51" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3781,7 +4543,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3796,19 +4558,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Filled in IELTS/TOEFL/GRE, references, tuition and scholarship amounts; flagged a cohort-year labeling ambiguity in the official deadline text.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3823,498 +4585,498 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Found the M2 ETE application window (10-20 Apr, recurring) and language/GRE/fee requirements — PhD entry is via M2 ETE only, not a standalone application.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>EUR-03</t>
+          <t>EUR-10</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
+          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Filled in deadline (31 Mar annually), GRE/reference requirements, and ZEW Cooperation Track funding — previously the least-detailed entry in the tracker.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>EUR-04</t>
+          <t>EUR-11</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Combined M.Sc. Economic Research / Doctoral Program — Bonn Graduate School of Economics (BGSE)</t>
+          <t>PhD in Economics and Finance — Bocconi University</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Confirmed the 2026-27 cycle (ordinary + FIS call) is fully closed and the 2027-28 cycle is not yet announced; added test-requirement and fee detail.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>EUR-05</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>PhD in Economics — CEMFI</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Confirmed deadlines unchanged; added admission requirement detail.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>EUR-06</t>
+          <t>ASA-02</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Master's in Economics — Barcelona School of Economics (BSE)</t>
+          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr) and fees; upgraded funding_status from Likely to Yes.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>EUR-07</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>PhD Program — Paris School of Economics (PSE)</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Site unreachable again this pass (DNS failure, confirmed via two methods); flagged an unconfirmed lead on a possible 2023 admission-policy change limiting PhD entry to internal Master's completers.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>EUR-08</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>PhD Programme in Economics — Stockholm University / IIES</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Located the correct department admissions page; found intake-cycle pattern, AO exam routes, and precise RePEc rank (#390).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>EUR-09</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MPhil + DPhil in Economics — University of Oxford</t>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Found university-wide test-score/fee requirements and admission-cycle pattern; department-specific PhD funding still unconfirmed.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>EUR-10</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Confirmed the imminent 31 Aug 2026 international scholarship deadline is still live; added RTP stipend figures; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>EUR-11</t>
+          <t>AUS-02</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>PhD in Economics and Finance — Bocconi University</t>
+          <t>Doctoral Program in Economics — University of Melbourne</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Found a reported Nov 2026 deadline and RTP stipend figures via search — official pages blocked automated fetches (HTTP 403), so flagged as lower confidence pending manual check.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>EUR-12</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Found an application-window pattern suggesting an imminent (~31 Aug 2026) integrated-pathway deadline; monash.edu blocked all direct fetches (HTTP 403), so figures are lower-confidence; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>PhD in Economics — University of Sydney</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Found general RTP scholarship deadlines (11 Sep / 18 Dec 2026); confirmed Sydney has no dedicated 'PhD in Economics' page — entry is via the general PhD degree; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>AUS-05</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
+          <t>PhD in Economics — UNSW Sydney</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Confirmed the EOI window remains closed with no new window announced; added program-structure and English-test detail.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ASA-03</t>
+          <t>EUR-13</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Hong Kong PhD Fellowship Scheme (HKPFS) — Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
+          <t>MRes/PhD in Economics — London School of Economics (LSE)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #16, funded via LSE PhD Studentships and ESRC studentships.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ASA-04</t>
+          <t>EUR-14</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
+          <t>MRes/PhD in Finance &amp; Economics — University of Warwick (Warwick Business School)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #37, fully funded (fee waiver + stipend) for all successful applicants.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-15</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>PhD in Economics (Zurich Graduate School of Economics) — University of Zurich</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #32, departmental scholarships from year 1 plus a competitive UBS Center Scholarship.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>EUR-16</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>PhD Programme in Economics — University of Copenhagen (Department of Economics)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #54, salaried PhD position under the Danish state academic-union pay scale (~EUR 4,150/month).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>ASA-08</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+          <t>PhD in Business (Economics track) — University of Hong Kong (Faculty of Business and Economics)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #106, guaranteed Postgraduate Scholarship funding (HK$19,135+/month) independent of the HKPFS scheme already tracked.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #71, RTP/UQGRSS stipend AUD $37,500/yr; flagged an imminent 31 Aug 2026 scholarship round.</t>
         </is>
       </c>
     </row>
@@ -4326,12 +5088,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>EUR-01</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics — University of Melbourne</t>
+          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -4353,12 +5115,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>EUR-02</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -4380,12 +5142,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>EUR-03</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -4407,20 +5169,560 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>EUR-04</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Combined M.Sc. Economic Research / Doctoral Program — Bonn Graduate School of Economics (BGSE)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>EUR-05</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>PhD in Economics — CEMFI</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>EUR-06</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Master's in Economics — Barcelona School of Economics (BSE)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>EUR-07</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>PhD Program — Paris School of Economics (PSE)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>EUR-08</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>PhD Programme in Economics — Stockholm University / IIES</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>EUR-09</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>MPhil + DPhil in Economics — University of Oxford</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>EUR-10</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>EUR-11</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>PhD in Economics and Finance — Bocconi University</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>EUR-12</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ASA-01</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ASA-02</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>ASA-03</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Hong Kong PhD Fellowship Scheme (HKPFS) — Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ASA-04</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>ASA-05</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>ASA-06</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>ASA-07</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>AUS-01</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>PhD in Economics — Australian National University (ANU)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>AUS-02</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Doctoral Program in Economics — University of Melbourne</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>AUS-03</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>PhD (Economics) — Monash Business School</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>AUS-04</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>PhD in Economics — University of Sydney</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
           <t>AUS-05</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>PhD in Economics — UNSW Sydney</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>Added (seed)</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>Initial research pass — program added to tracker.</t>
         </is>

</xml_diff>

<commit_message>
Econ ledger update 2026-08-29: 5 added, 8 updated, 3 reminder flags
5 new funded programs (VGSE Vienna, Tilburg, KU Leuven, Berlin School of
Economics, CUHK). Filled gaps on 4 Asian entries (NTU, UTokyo, Hitotsubashi,
SNU). Reconfirmed 3 imminent Australian deadlines (ANU, Monash, UQ) and
tripped their 7-day reminder flags. Telegram sync already posted these
changes live to @EconGradAlerts.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/EconGradAlert/data/tracker.xlsx
+++ b/apps/EconGradAlert/data/tracker.xlsx
@@ -438,7 +438,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last full research pass: 2026-08-23</t>
+          <t>Last full research pass: 2026-08-29</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Program count: 30</t>
+          <t>Program count: 35</t>
         </is>
       </c>
     </row>
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y31"/>
+  <dimension ref="A1:Y36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2717,7 +2717,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>EUR-17</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2732,373 +2732,373 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>National University of Singapore (NUS)</t>
+          <t>Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>#120</t>
+          <t>~#192 (University of Vienna, Institute for Economics) — search-derived, not independently verified against the live RePEc table</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Vienna</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>https://fass.nus.edu.sg/ecs/doctor-of-philosophy-economics/</t>
+          <t>https://www.vgse.at/</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Not mentioned (standard faculty requirement applies)</t>
+          <t>7.0 minimum</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Not mentioned (standard faculty requirement applies)</t>
+          <t>100 iBT minimum (internet-based)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Not mentioned on this page</t>
+          <t>No formal minimum published; admitted students typically score Q&gt;=164 (not officially confirmed)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Non-English-medium graduates may need to take a Graduate English Course; good undergraduate honours degree (first class or high 2:1 equivalent) or Master's, in economics or another quantitative subject</t>
+          <t>Strong BA/MA grades expected; background in micro/macro/econometrics required; motivation letter, research proposal, and an 'Indication of Willingness to Supervise' form from a VGSE faculty member all required</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>October (winter term)</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Early: 30 September 2026; Main: 1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
+          <t>Two admission rounds reported — roughly 1 Dec-15 Feb and 1 Mar-30 Apr on one page, vs. a single 1 Feb-15 Jun window on the VGSE-specific page; exact current-cycle dates are inconsistent across the university's own sources, recommend a manual spot-check</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>soon</t>
+          <t>later</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>2 (academic)</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
+          <t>Not found — likely none</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>Not detailed (fully funded — see funding)</t>
+          <t>Not disclosed on pages checked; Austrian public-university PhDs are typically low/near-free for EU students, unconfirmed for non-EU</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Yes — all admitted students</t>
+          <t>Yes — competitive</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>Full financial support (fees + living expenses) for 5 years: NUS Research Scholarship (years 1-4), department funding (year 5), plus research/travel allowance.</t>
+          <t>Program is funded via an Austrian Science Fund (FWF) grant; successful applicants receive funded PhD positions at the University of Vienna. Exact stipend amount not disclosed on public pages — confirm directly with VGSE.</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>Confirmed deadlines unchanged; added admission requirement detail</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; contact econ-phd@nus.edu.sg for specifics</t>
+          <t>New find Aug 2026; admission-round dates are inconsistent across the university's own pages — verify the current-cycle deadline directly before relying on it; stipend amount unconfirmed.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>EUR-18</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MPhil/PhD</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics</t>
+          <t>PhD in Economics</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Hong Kong University of Science and Technology (HKUST)</t>
+          <t>Tilburg University (CentER Graduate School)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>#287</t>
+          <t>~#24 (Tilburg School of Economics and Management) — search-derived, not independently verified</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Hong Kong (China)</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Tilburg</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>https://econ.hkust.edu.hk/programs-n-courses/mphd/mphd-admission</t>
+          <t>https://www.tilburguniversity.edu/research/economics-and-management/graduate-school/phd-economics</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>6.5 overall, no subscore below 5.5 (university-wide standard; waived if English-medium/first-language English)</t>
+          <t>Not confirmed this pass (official financial-matters page returned HTTP 403 to direct fetch)</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>iBT 80 / pBT 550 / Revised PBT 60 (university-wide standard)</t>
+          <t>Not confirmed this pass (same 403 caveat)</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Required ("satisfactory score")</t>
+          <t>Non-EU applicants must submit a recent GRE or GMAT score; EU applicants may substitute 24 ECTS of quantitative coursework instead</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Conditional offers require official documents by end of July</t>
+          <t>Academic/Research Master's in economics or econometrics with an excellent GPA expected; the PhD is structured as a paid employment contract, not a fee-paying admission</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Fall semester</t>
+          <t>Typically September (standard Dutch academic year; not independently confirmed this pass)</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
+          <t>Not firmly confirmed — PhD vacancies are posted and filled on a rolling basis rather than a single fixed annual deadline; check the vacancies page directly</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>soon</t>
+          <t>tba</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not confirmed this pass</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>HK$180, non-refundable</t>
+          <t>Not found — likely none (PhD is an employment contract, not a fee-paying admission)</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>HK$47,000/year (2026/27 rate, full-time or part-time)</t>
+          <t>None — PhD candidates are salaried university employees, no tuition charged</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes — salaried employee position</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>Postgraduate Studentship (PGS): HK$229,620/year (2025/26 rate); recipients serve as Graduate Teaching Assistants. HKUST RedBird PhD Award stacks with HKPFS: Recruitment Award HK$40,000 (year 1) + Academic Excellence Award HK$20,000/year (later years). Conference &amp; Travel Allowance ~HK$14,200/year for HKPFS holders. Also cross-reference Hong Kong PhD Fellowship Scheme (ASA-03).</t>
+          <t>PhD candidates are Tilburg University employees on a gross monthly salary reported at ~EUR 2,750 (year 1) rising to ~EUR 3,500 (year 4), plus a May holiday allowance and a November year-end bonus. Reported via search only — the official financial-matters page returned HTTP 403 to direct fetch, recommend verifying directly.</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr), fees, and IELTS/TOEFL standards; upgraded funding_status from Likely to Yes</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026</t>
+          <t>New find Aug 2026; official site blocked automated fetches (HTTP 403) on several pages, so deadline, exact salary, and requirements rely on search snippets only — verify directly before relying on them.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ASA-03</t>
+          <t>EUR-19</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PhD (Fellowship, cross-university)</t>
+          <t>PhD</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Hong Kong PhD Fellowship Scheme (HKPFS)</t>
+          <t>Doctoral Programme in Economics</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
+          <t>KU Leuven (Faculty of Economics and Business)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Varies by host university (scheme spans multiple HK institutions)</t>
+          <t>~#40 (KU Leuven, Faculteit Economie en Bedrijfswetenschappen) — search-derived, not independently verified</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Hong Kong (China)</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Leuven</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>https://www.gs.cuhk.edu.hk/admissions/scholarships-fees/hkpfs</t>
+          <t>https://feb.kuleuven.be/research/economics/PHD/overview</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules (set by individual dept/program)</t>
+          <t>7.0 minimum (general KU Leuven PhD policy, not confirmed program-specific)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules (set by individual dept/program)</t>
+          <t>90 iBT minimum (internet-based; same caveat as IELTS)</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules (set by individual dept/program)</t>
+          <t>Not mentioned as a requirement</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Apply via 2 parallel channels: RGC website (choose up to 2 programmes) AND university's own online system, quoting HKPFS reference number. Selection on academic excellence, research potential, communication, leadership.</t>
+          <t>Direct entry requires a completed Research Master's in economics or a related field; applicants with only an initial (non-research) Master's can enter via the MASE pre-doctoral track first</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Typically September (Fall)</t>
+          <t>September; new PhD vacancies posted each December</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>1 December 2026, 12:00 noon HKT (RGC) / 11:59pm HKT (university, e.g. CUHK)</t>
+          <t>Rolling, per individual vacancy posting rather than one fixed annual date — one past round cited a 31 Jan closing (2025 cohort) for illustration only; check the current vacancy list directly</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>soon</t>
+          <t>tba</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>Not specified in scheme rules</t>
+          <t>Not specified in sources checked</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not found</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>Waived (see funding)</t>
+          <t>EUR 461/year (registration year and defence year only; no fee in the years between)</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>Yes — major fellowship</t>
+          <t>Yes — competitive</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>~HK$1.81 million total (~US$232,400): stipend HK$344,400/yr (~US$44,200), conference/travel HK$14,400/yr, tuition waiver up to HK$198,000, lodging award up to HK$100,000, first-year hostel waiver.</t>
+          <t>PhD positions funded for up to 4 years (initial 12-month contract, extended on positive evaluation). Separately, IRO Doctoral Scholarships for students from developing countries include a tuition waiver, a monthly stipend of EUR 1,000-1,415, a EUR 200/month allowance, and social security coverage.</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; this is a cross-institution scheme, not a single program — apply through chosen university's Economics dept</t>
+          <t>New find Aug 2026; deadline is vacancy-by-vacancy rather than a single annual date — check the live vacancy list before relying on any specific date.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ASA-04</t>
+          <t>EUR-20</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3108,124 +3108,124 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>PhD Program (Economics track)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Nanyang Technological University (NTU Singapore)</t>
+          <t>Berlin School of Economics (BSE) — joint doctoral school across multiple Berlin-area institutions</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>#253</t>
+          <t>~#164 (Humboldt-Universität zu Berlin, Wirtschaftswissenschaftliche Fakultät, as coordinating institution) — search-derived; BSE is a multi-institution consortium so this reflects only the host department, not the consortium as a whole</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>https://www.ntu.edu.sg/education/graduate-programme/ph.d.-in-economics</t>
+          <t>https://berlinschoolofeconomics.de/phd-program</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>7.0 minimum (preferred)</t>
+          <t>Recommended but not mandatory for non-native speakers who hold an English-taught degree</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>105 minimum</t>
+          <t>Same as IELTS field — recommended, not mandatory if prior degree was English-taught</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Not mandatory, but scores considered if submitted; recommended for non-Singapore-university degree holders</t>
+          <t>Recommended, not mandatory (institution code 3853); no fixed minimum published</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Scores must be within 2 years of application; exemptions for native speakers / English-medium degree holders</t>
+          <t>Joint doctoral school spanning multiple Berlin-area research institutions (incl. Humboldt-Universität zu Berlin, Freie Universität Berlin, TU Berlin, European University Viadrina, University of Potsdam, ESMT Berlin, Hertie School, WZB, and affiliated economic-research institutes); Master's in economics/business or a related quantitative field required; 2-page motivation letter, CV, and transcripts</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>October annually</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Not specified on this page — contact ac-sss-ge@ntu.edu.sg</t>
+          <t>~15 January annually (confirmed for the 2026 cohort; reconfirm the exact date closer to the next cycle)</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>tba</t>
+          <t>later</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>2 (academic, submitted directly by referees via the application portal)</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>None found; admitted students pay a general semester fee of ~EUR 300-350 (standard German-university Semesterbeitrag, not program-specific)</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>Not specified (MOE-subsidised place)</t>
+          <t>None — no tuition fees</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes — funded across both phases</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>MOE-subsidised programme; Nanyang Research Scholarship available for qualifying students.</t>
+          <t>Qualification phase (~3 semesters): monthly stipend of EUR 1,650, plus a family allowance if applicable. Dissertation phase (~3 years): funded via employment at a BSE member institution.</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; deadline needs manual confirmation</t>
+          <t>New find Aug 2026; joint doctoral school across multiple Berlin institutions rather than a single university — Economics is one of several eligible fields.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3235,17 +3235,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD)</t>
+          <t>PhD in Economics</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>University of Tokyo</t>
+          <t>National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>#110</t>
+          <t>#120</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -3255,77 +3255,77 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Tokyo</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>https://www.gaia.e.u-tokyo.ac.jp/utipe/</t>
+          <t>https://fass.nus.edu.sg/ecs/doctor-of-philosophy-economics/</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not mentioned (standard faculty requirement applies)</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not mentioned (standard faculty requirement applies)</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not mentioned on this page</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>English-taught international program; site (gaia.e.u-tokyo.ac.jp) unreachable again this pass — DNS resolution failure confirmed via two independent fetch methods, same issue as prior pass</t>
+          <t>Non-English-medium graduates may need to take a Graduate English Course; good undergraduate honours degree (first class or high 2:1 equivalent) or Master's, in economics or another quantitative subject</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not specified on this page</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Not yet confirmed — needs manual check</t>
+          <t>Early: 30 September 2026; Main: 1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>tba</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not detailed (fully funded — see funding)</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>Likely (MEXT scholarship-eligible — common for UTokyo international programs)</t>
+          <t>Yes — all admitted students</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>Not confirmed this pass — MEXT (Japanese government) scholarship route is commonly available for this program; needs verification.</t>
+          <t>Full financial support (fees + living expenses) for 5 years: NUS Research Scholarship (years 1-4), department funding (year 5), plus research/travel allowance.</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
@@ -3340,39 +3340,39 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>Site unreachable again (DNS failure) — no field data updated; flagged an unconfirmed lead on a possible admission-policy change</t>
+          <t>Confirmed deadlines unchanged; added admission requirement detail</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>INCOMPLETE — prioritise for next refresh. Unconfirmed search snippets suggest UTIPE's PhD admission policy changed circa 2023 to require completing UTIPE's own Master's program first (may no longer accept direct external PhD applicants) — not verified against the primary source, needs a manual check.</t>
+          <t>Seed entry Aug 2026; contact econ-phd@nus.edu.sg for specifics</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>ASA-02</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>MPhil/PhD</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD)</t>
+          <t>MPhil/PhD in Economics</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Hitotsubashi University</t>
+          <t>Hong Kong University of Science and Technology (HKUST)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>#390 (confirmed still outside global top 300)</t>
+          <t>#287</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -3382,77 +3382,77 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Hong Kong (China)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Tokyo (Kunitachi)</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>https://www.econ.hit-u.ac.jp/eng/page/graduate/admission.html</t>
+          <t>https://econ.hkust.edu.hk/programs-n-courses/mphd/mphd-admission</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Not stated (page mentions TOEFL/TOEIC only)</t>
+          <t>6.5 overall, no subscore below 5.5 (university-wide standard; waived if English-medium/first-language English)</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>TOEFL or TOEIC score required as part of application materials; specific minimum score not stated</t>
+          <t>iBT 80 / pBT 550 / Revised PBT 60 (university-wide standard)</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
+          <t>Required ("satisfactory score")</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Two intakes/year (Spring and Autumn); international applicants without a Hitotsubashi Master's apply via an AO exam route — either general AO (2+ years work experience post-master's) or AO for international applicants with a Master's from outside Japan; admission mainly via submitted documents, interview may follow (online option for overseas applicants)</t>
+          <t>Conditional offers require official documents by end of July</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Spring or Autumn intake (two cycles/year)</t>
+          <t>Fall semester</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Applications open ~October (for the following Spring start) and ~April (for the following Autumn start); exact day-level deadlines are issued per-cycle in a separate department announcement, not found this pass</t>
+          <t>1 December 2026 (recurring annual pattern, applied to the upcoming cycle)</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>tba</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>At least 1 recommendation letter required (exact number not specified)</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>HK$180, non-refundable</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>HK$47,000/year (2026/27 rate, full-time or part-time)</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>Likely (MEXT scholarship-eligible)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>MEXT scholarship route confirmed to exist, administered via a separate central international-office page (requires embassy/consulate preliminary candidacy). No department-specific stipend/assistantship figures found.</t>
+          <t>Postgraduate Studentship (PGS): HK$229,620/year (2025/26 rate); recipients serve as Graduate Teaching Assistants. HKUST RedBird PhD Award stacks with HKPFS: Recruitment Award HK$40,000 (year 1) + Academic Excellence Award HK$20,000/year (later years). Conference &amp; Travel Allowance ~HK$14,200/year for HKPFS holders. Also cross-reference Hong Kong PhD Fellowship Scheme (ASA-03).</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
@@ -3467,39 +3467,39 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>Located the correct department admissions page (previous link was a generic university page); found intake-cycle pattern, AO exam routes, and precise RePEc rank (#390)</t>
+          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr), fees, and IELTS/TOEFL standards; upgraded funding_status from Likely to Yes</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>Partially complete — exact per-cycle deadline dates and funding figures still needed; prioritise for next refresh</t>
+          <t>Seed entry Aug 2026</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>ASA-03</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PhD</t>
+          <t>PhD (Fellowship, cross-university)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD)</t>
+          <t>Hong Kong PhD Fellowship Scheme (HKPFS)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Seoul National University (SNU)</t>
+          <t>Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>#189</t>
+          <t>Varies by host university (scheme spans multiple HK institutions)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -3509,77 +3509,77 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Hong Kong (China)</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Seoul</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>https://en.snu.ac.kr/admission</t>
+          <t>https://www.gs.cuhk.edu.hk/admissions/scholarships-fees/hkpfs</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>6.0 minimum (university-wide standard)</t>
+          <t>Not specified in scheme rules (set by individual dept/program)</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>iBT 80, or TEPS 551 (university-wide standard, alternative to IELTS)</t>
+          <t>Not specified in scheme rules (set by individual dept/program)</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Not required (no GRE requirement found in central admissions materials)</t>
+          <t>Not specified in scheme rules (set by individual dept/program)</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>University-wide scholarships identified; department-level participation not yet confirmed</t>
+          <t>Apply via 2 parallel channels: RGC website (choose up to 2 programmes) AND university's own online system, quoting HKPFS reference number. Selection on academic excellence, research potential, communication, leadership.</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Typically September (Fall)</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>University-wide pattern: Fall-intake applications open ~early March (2026 Fall: 3-5 Mar); Spring-intake applications open ~early July (2027 Spring: 6-9 Jul) — both 2026 cycles already closed; 2027 Fall cycle not yet announced. Department-specific PhD deadline still not separately confirmed.</t>
+          <t>1 December 2026, 12:00 noon HKT (RGC) / 11:59pm HKT (university, e.g. CUHK)</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>later</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Not specified in scheme rules</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>KRW 90,000 (no fee waivers offered)</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>Not yet confirmed</t>
+          <t>Waived (see funding)</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>Likely (university-wide scholarships)</t>
+          <t>Yes — major fellowship</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>Global Korea Scholarship: full tuition (6 semesters) + ~1.4M KRW/month + airfare (Korean language req., TOPIK 3; deadline ~February). SNU President Fellowship: full tuition + 1.5-2M KRW/month. Grad Scholarship for Excellent Foreign Students: full tuition (4 semesters) + 500K KRW/month min. Dept-level applicability not yet confirmed — search turned up only informal/unofficial claims (e.g. individual professors self-funding RAs from grants), not an official department statement.</t>
+          <t>~HK$1.81 million total (~US$232,400): stipend HK$344,400/yr (~US$44,200), conference/travel HK$14,400/yr, tuition waiver up to HK$198,000, lodging award up to HK$100,000, first-year hostel waiver.</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
@@ -3589,24 +3589,24 @@
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>Found university-wide test-score/fee requirements and admission-cycle pattern; department-specific PhD funding still unconfirmed</t>
+          <t>Added (seed)</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>Department-level Economics PhD funding not yet confirmed — university-wide scholarships only; prioritise for next refresh</t>
+          <t>Seed entry Aug 2026; this is a cross-institution scheme, not a single program — apply through chosen university's Economics dept</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ASA-08</t>
+          <t>ASA-04</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3616,17 +3616,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>PhD in Business (Economics track)</t>
+          <t>PhD in Economics</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>University of Hong Kong (Faculty of Business and Economics)</t>
+          <t>Nanyang Technological University (NTU Singapore)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>#106</t>
+          <t>#253</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3636,47 +3636,47 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Hong Kong (China)</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>https://phd.hkubs.hku.hk/admissions/admission-application-and-tuition-fee</t>
+          <t>https://www.ntu.edu.sg/education/graduate-programme/ph.d.-in-economics</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Academic overall 6.5, all subtests &gt;= 6.0 (waived if prior degree was taught in English)</t>
+          <t>7.0 minimum (preferred)</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>iBT &gt;= 85</t>
+          <t>105 minimum</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>GRE or GMAT required, score &lt;5 years old (institution codes: GRE 2482, GMAT FS2-WL-48)</t>
+          <t>Not mandatory, but scores considered if submitted; recommended for applicants without a degree from an autonomous university</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Bachelor's with first-class honours (or equivalent), or Bachelor's + Master's from a recognized university; 3-year track with a research Master's, 4-year track without one; Economics is one of six FBE PhD fields</t>
+          <t>Scores must be within 2 years of application; exemptions for native speakers / English-medium degree holders; 2 referee reports required</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Fall semester, normally September (matriculates once a year)</t>
+          <t>Two intakes/year: August (main) and January</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Applications open 1 September; Main Round closes 1 December (recurring annual cycle; late applications considered only if places remain)</t>
+          <t>August intake: applications open 1 Oct-15 Nov (results Mar-May); January intake: applications open 1 Jun-31 Jul (results Nov-Dec) — recurring annual pattern, confirmed via direct official fetch</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
@@ -3686,17 +3686,17 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>2 (academic referee reports, submitted directly by referees)</t>
+          <t>2 (referee reports)</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>HK$600 (paid online via HKU Graduate School application system)</t>
+          <t>S$50</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>HK$49,500/year (2027-28 rate) for full-time PhD — typically waived/covered for scholarship holders</t>
+          <t>Not specified (MOE-subsidised place)</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
@@ -3706,34 +3706,34 @@
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>Standard Postgraduate Scholarship (PGS) pays HK$19,135/month (rising to HK$19,655/month once candidature is confirmed), available to essentially all admitted PhD students regardless of HKPFS status. HKPFS awardees instead receive HK$28,700/month plus HK$14,400/year travel allowance for up to 3 years.</t>
+          <t>MOE-subsidised programme; funded via Nanyang President's Graduate Scholarship or Nanyang Research Scholarship, which carries Graduate Assistantship Programme (GAP) teaching/research duties.</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Confirmed application windows, referee/fee requirements via direct official fetch; urgency upgraded from tba to soon</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>Distinct from the cross-institution HKPFS scheme already tracked (ASA-03) — nearly all admitted PhD students get baseline PGS funding here even without winning HKPFS, a broader guarantee than HKPFS alone.</t>
+          <t>Seed entry Aug 2026; tuition fee figure still not found</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3743,97 +3743,97 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>International Program in Economics (PhD)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Australian National University (ANU)</t>
+          <t>University of Tokyo</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>#124</t>
+          <t>#110</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Canberra</t>
+          <t>Tokyo</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>https://cbe.anu.edu.au/study/graduate-research-programs/doctor-philosophy-phd/phd-economics</t>
+          <t>https://www.gaia.e.u-tokyo.ac.jp/utipe/</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>6.5 overall (no band below 6.0)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>570 (paper-based; essay ≥4.5)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Mandatory (code 7833); exempt if ANU Econ Honours/Masters</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Pre-PhD summer course required, Jan-Feb, arriving 4-6 weeks before semester</t>
+          <t>English-taught international program; site (gaia.e.u-tokyo.ac.jp) unreachable for a third consecutive pass — DNS resolution failure confirmed again via independent fetch attempts. As of April 2023, UTIPE PhD applicants are generally required to first complete UTIPE's own Master's program and be admitted to candidacy; direct external PhD entry is closed except for applicants with 2+ years of research experience at a university/research institute abroad (following 16 years of foreign schooling), who may be recognized as equivalent to a Master's holder and apply directly. Corroborated via search snippets quoting the official admission/FAQ pages, not a direct primary-source fetch.</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>February (Semester 1); Semester 2 entry possible (July)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>For Feb 2027 start: international scholarship applicants before 31 Aug 2026 (imminent), standard before 31 Oct 2026; Sem 2 entry before 31 Mar</t>
+          <t>Not yet confirmed — needs manual check</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>urgent</t>
+          <t>tba</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Likely (MEXT scholarship-eligible — common for UTokyo international programs)</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>Australian Government RTP Stipend: AUD $39,069/year (2026 full-time base rate, ANU-wide), paid fortnightly, up to 3.5 years. Some HDR supplementary scholarships add AUD $7,000/year on top, for up to 3 years. Domestic candidates pay no tuition (RTP-covered); international candidates can compete for HDR Fee Remission Merit Scholarships covering up to 4 years.</t>
+          <t>Not confirmed this pass — MEXT (Japanese government) scholarship route is commonly available for this program; needs verification.</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
@@ -3843,24 +3843,24 @@
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>Confirmed the 31 Aug 2026 international scholarship deadline is still live (verified directly on program page); added RTP stipend figures; set 30-day reminder flag</t>
+          <t>Corroborated (via search snippets of official FAQ/admission pages) that UTIPE has restricted direct external PhD entry since April 2023 to applicants with 2+ years research experience abroad; site itself remains unreachable (DNS failure, third consecutive pass)</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026 — international scholarship deadline is imminent (8 days away as of this update)</t>
+          <t>INCOMPLETE — prioritise for next refresh, though the site has now failed to resolve on three consecutive passes; consider a manual browser check. The 2023 admission-policy restriction is now corroborated by multiple search snippets quoting the official pages, but still not confirmed via a direct primary-source fetch.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3870,67 +3870,67 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics</t>
+          <t>Graduate School of Economics (PhD)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>University of Melbourne</t>
+          <t>Hitotsubashi University</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>#151</t>
+          <t>#390 (confirmed still outside global top 300)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Melbourne</t>
+          <t>Tokyo (Kunitachi)</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>https://study.unimelb.edu.au/find/courses/graduate/doctoral-program-in-economics/how-to-apply/</t>
+          <t>https://www.econ.hit-u.ac.jp/eng/page/graduate/admission.html</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>7.0 overall (7.0 writing, no band below 6.0)</t>
+          <t>Not stated (page mentions TOEFL/TOEIC only)</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>94 iBT (W27/S18/R13/L13)</t>
+          <t>TOEFL or TOEIC score required as part of application materials; specific minimum score not stated</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Not mentioned in entry requirements</t>
+          <t>Not mentioned</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>PTE Academic 72+ (written 75+); CAE 185+ also accepted; 5-year program (2 coursework + 3 research)</t>
+          <t>Two intakes/year (Spring and Autumn); international applicants without a Hitotsubashi Master's apply via an AO exam route — either general AO (2+ years work experience post-master's) or AO for international applicants with a Master's from outside Japan; admission mainly via submitted documents, interview may follow (online option for overseas applicants)</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>March intake</t>
+          <t>Spring or Autumn intake (two cycles/year)</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>March 2027 intake deadline reported as 30 November 2026 — found via search summary only; the official how-to-apply/key-dates pages returned HTTP 403 on every direct fetch attempt this pass, so this date is unconfirmed by primary source and should be manually verified</t>
+          <t>Spring intake: document submission window ~14-17 Oct annually (confirmed for the Spring 2026 cohort: 14-17 Oct 2025, results ~11 Nov 2025), so the next window is expected ~mid-Oct 2026 for Spring 2027 entry. Autumn intake: opens ~April, exact window not confirmed this pass.</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -3940,27 +3940,27 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>At least 1 recommendation letter required (AO exam route requires an English-language Letter of Recommendation); exact number for other routes not specified</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
+          <t>~JPY 30,000 reported (university-wide general graduate-school figure, not confirmed Economics-specific)</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>Not detailed — full tuition fee waiver reported (see funding)</t>
+          <t>~JPY 535,800/year reported (university-wide figure, not confirmed Economics-PhD-specific)</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Likely (MEXT scholarship-eligible)</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>Australian Government Research Training Program (RTP) funded places available: RTP stipend reported at AUD $39,500/year (2026 rate) plus full tuition fee waiver and AUD $15,000 research/conference travel funding for confirmed PhD candidates (unconfirmed by primary source — see deadline note). Program structure: 2-year Master of Commerce coursework + 3-year PhD.</t>
+          <t>MEXT scholarship route confirmed to exist, administered via a separate central international-office page (requires embassy/consulate preliminary candidacy). No department-specific stipend/assistantship figures found.</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">
@@ -3970,24 +3970,24 @@
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>Found a reported deadline and funding figures via search, but could not confirm via direct page fetch (403 blocked) — flagged as lower confidence</t>
+          <t>Found the Spring-intake AO-exam submission window (~14-17 Oct, recurring annually) and fee figures via search corroboration (official PDF/page blocked direct fetch by an SSL certificate error); urgency upgraded from tba to soon</t>
         </is>
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; unimelb.edu.au pages returned HTTP 403 to automated fetches this pass — recommend a manual browser check before relying on the reported 30 Nov 2026 deadline</t>
+          <t>Partially complete — fee figures are university-wide, not Economics-PhD-confirmed; exact Autumn-intake window still needed</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3997,97 +3997,97 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PhD (Economics)</t>
+          <t>Department of Economics (PhD)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Monash Business School</t>
+          <t>Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>#46</t>
+          <t>#189</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Melbourne (Clayton)</t>
+          <t>Seoul</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>https://www.monash.edu/business/research/phd-programs/scholarships-and-fees</t>
+          <t>https://en.snu.ac.kr/admission</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>7.0 minimum reported (third-party source, not confirmed on official Monash page — page returned HTTP 403 to direct fetch)</t>
+          <t>6.0 minimum (university-wide standard)</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>94 minimum reported (same caveat as IELTS — unconfirmed by primary source)</t>
+          <t>iBT 80, or TEPS 551 (university-wide standard, alternative to IELTS)</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>Not required (no GRE requirement found in central admissions materials)</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Multiple named scholarships stack with base RTP/Monash funding</t>
+          <t>University-wide scholarships identified; department-level participation not yet confirmed</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>Two pathways found (via search — official pages returned HTTP 403 to direct fetch, unconfirmed by primary source): Integrated PhD program (Master of Commerce + PhD), Feb/Semester-1 entry — applications open 1 Jul-31 Aug (closing imminently); Jul/Semester-2 entry — applications open 1 Dec-1 Feb. Separately, general Graduate Research Scholarship rounds: international Round 1 closes 31 Mar, Round 3 closes ~31 Jul/31 Aug; domestic Round 2 closes 31 May, Round 4 closes 31 Oct.</t>
+          <t>University-wide pattern: Fall-intake applications open ~early March (2026 Fall: 3-5 Mar); Spring-intake applications open ~early July (2027 Spring: 6-9 Jul) — both 2026 cycles already closed; 2027 Fall cycle not yet announced. Department-specific PhD deadline still not separately confirmed.</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>urgent</t>
+          <t>later</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>KRW 90,000 (no fee waivers offered)</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>International ~AUD $38,900/yr, domestic ~AUD $37,100/yr reported (third-party aggregator source, not confirmed by official Monash page)</t>
+          <t>Not yet confirmed</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Likely (university-wide scholarships only)</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>Donald Cochrane Scholarship: AUD 10,000/yr x 3.5yrs (3 awarded/yr). Dean's Excellence Award: up to AUD 5,000/yr top-up (10/yr). Graduate Research Scholarship: AUD 41,000/yr tuition (~12/yr). Plus university-wide Monash Graduate Scholarship / RTP places.</t>
+          <t>Global Korea Scholarship: full tuition (6 semesters) + ~1.4M KRW/month + airfare (Korean language req., TOPIK 3; deadline ~February). SNU President Fellowship: full tuition + 1.5-2M KRW/month. Grad Scholarship for Excellent Foreign Students: full tuition (4 semesters) + 500K KRW/month min. Confirmed via direct fetch of the Department of Economics' own PhD page: no department-specific funding scheme exists — funding runs entirely through the university-wide scholarships above.</t>
         </is>
       </c>
       <c r="V28" t="inlineStr">
@@ -4097,24 +4097,24 @@
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>Found application-window pattern suggesting an imminent (~31 Aug) integrated-pathway deadline, plus fee/test figures — all via search snippets/third-party sites since monash.edu returned HTTP 403 on every direct fetch attempt; set 30-day reminder flag pending confirmation</t>
+          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; admissions and funding run entirely through the university-wide portal and scholarships</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; monash.edu blocked all automated fetches this pass (scholarships-and-fees, apply, and program pages all 403'd) — every figure in this update is lower-confidence (search snippets/third-party aggregator only) and needs a manual browser check, especially the reported 31 Aug 2026 integrated-pathway deadline</t>
+          <t>Confirmed (Aug 2026) that Economics PhD funding at SNU is university-wide only, with no departmental top-up scheme; department page exists but defers entirely to the central international-admissions portal for deadlines/fees</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>ASA-08</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -4124,87 +4124,87 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PhD in Economics</t>
+          <t>PhD in Business (Economics track)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>University of Sydney</t>
+          <t>University of Hong Kong (Faculty of Business and Economics)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>#87</t>
+          <t>#106</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Hong Kong (China)</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Sydney</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>https://www.sydney.edu.au/scholarships/</t>
+          <t>https://phd.hkubs.hku.hk/admissions/admission-application-and-tuition-fee</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Not specified at general program level</t>
+          <t>Academic overall 6.5, all subtests &gt;= 6.0 (waived if prior degree was taught in English)</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Not specified at general program level</t>
+          <t>iBT &gt;= 85</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Not mentioned</t>
+          <t>GRE or GMAT required, score &lt;5 years old (institution codes: GRE 2482, GMAT FS2-WL-48)</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Example named scholarship seen (topic-restricted, econ conflict/ag markets) — general program funding likely via RTP. Material finding: Sydney has no dedicated 'PhD in Economics' program page — the Economics coursework handbook explicitly states it "does not include a research component and thus does not provide a pathway to higher degree by research (e.g. PhD) studies." PhD study is pursued via the general Doctor of Philosophy degree with a nominated Economics supervisor/discipline, not a single named landing page.</t>
+          <t>Bachelor's with first-class honours (or equivalent), or Bachelor's + Master's from a recognized university; 3-year track with a research Master's, 4-year track without one; Economics is one of six FBE PhD fields</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Not specified on this page</t>
+          <t>Fall semester, normally September (matriculates once a year)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>General Research Training Program (RTP) scholarship rounds for 2027 entry (found via search, not a directly-fetched dedicated Economics PhD page): Research Period 1 &amp; 2 — deadline 11 September 2026; Research Period 3 &amp; 4 — deadline 18 December 2026.</t>
+          <t>Applications open 1 September; Main Round closes 1 December (recurring annual cycle; late applications considered only if places remain)</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>urgent</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>1 (for named scholarship example; general program may differ)</t>
+          <t>2 (academic referee reports, submitted directly by referees)</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>HK$600 (paid online via HKU Graduate School application system)</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>HK$49,500/year (2027-28 rate) for full-time PhD — typically waived/covered for scholarship holders</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
@@ -4214,12 +4214,12 @@
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>RTP-style stipend scholarships ~AUD 41,753/yr (base AUD 37,207 + top-up), up to 3 years, seen via School of Economics named scholarship. General RTP funding also available for the PhD program broadly.</t>
+          <t>Standard Postgraduate Scholarship (PGS) pays HK$19,135/month (rising to HK$19,655/month once candidature is confirmed), available to essentially all admitted PhD students regardless of HKPFS status. HKPFS awardees instead receive HK$28,700/month plus HK$14,400/year travel allowance for up to 3 years.</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="W29" t="inlineStr">
@@ -4229,19 +4229,19 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>Found general RTP scholarship round deadlines (11 Sep / 18 Dec 2026); confirmed there is no dedicated Sydney 'PhD in Economics' page — entry is via the general PhD degree with an Economics supervisor; set 30-day reminder flag</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026; needs a general (non-topic-restricted) funding page check; no dedicated Economics-specific PhD admissions page exists at Sydney</t>
+          <t>Distinct from the cross-institution HKPFS scheme already tracked (ASA-03) — nearly all admitted PhD students get baseline PGS funding here even without winning HKPFS, a broader guarantee than HKPFS alone.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AUS-05</t>
+          <t>ASA-09</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -4256,239 +4256,874 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>UNSW Sydney</t>
+          <t>Chinese University of Hong Kong (CUHK), Department of Economics</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>#80</t>
+          <t>~#369 — search-derived, not independently verified against the live RePEc table</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Hong Kong (China)</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Sydney</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://www.unsw.edu.au/business/study-with-us/postgraduate-research/phd-degrees/doctor-philosophy-phd-economics</t>
+          <t>https://admission.econ.cuhk.edu.hk/pg/phd-economics/</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Not listed on this page (exemptions for AU/CA/UK/US/NZ citizens); non-English-speaking-country applicants need IELTS/TOEFL/PTE/Cambridge or the UNSW Global English Course</t>
+          <t>Academic overall 6.5</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Not listed on this page — see IELTS field for alternatives</t>
+          <t>79 iBT (or 4.5-6.0 Home Edition) — see IELTS field for alternatives (GMAT Verbal &gt;=21, or a degree from an English-medium institution, also accepted)</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Optional but recommended overall; one source indicates GRE may be specifically required for the Economics stream — this conflicts with the general 'optional' language elsewhere and needs manual confirmation</t>
+          <t>Required (institution code 3153, department code 1801); no published hard cutoff, but absence of a score disadvantages applicants</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Alternative English tests: PTE, Cambridge, or UNSW Global English Course. Program begins with a 1-year Master of Pre-Doctoral Business Studies, followed by 3-3.5 years of doctoral research; direct entry to the 3-year PhD is possible for candidates with first-class Honours/Master's plus independent funding (Stream 2).</t>
+          <t>Master's in economics or a related field with a strong math/stats background expected; strong bachelor's-only applicants can also apply with sufficient research potential. Official transcripts, degree certificates, a 5-page research proposal and/or working papers, resume, and typically an interview all required</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Term 1 – February</t>
+          <t>Fall intake (standard)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Confirmed still closed as of 23 Aug 2026 (verified directly on program page): EOI window opened 20 March 2026, closed 15 August 2026, no newer/next EOI window posted. Note: a separate 26 August 2026 formal-application deadline exists, but it applies only to candidates already invited to apply from the closed EOI round, not to new applicants.</t>
+          <t>Applications open 1 Sept 2026; HKPFS-track deadline 1 Dec 2026 (11:59am); non-HKPFS deadline 1 Dec 2026 (11:59pm); referee letters due by 4 Dec 2026</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>soon</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>3 confidential recommendation letters</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>HK$500 per programme</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>Not detailed (fully funded — see funding)</t>
+          <t>HK$47,000 (2026/27) / HK$49,500 (2027/28)</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>Yes — all admitted students</t>
+          <t>Yes — guaranteed assistantship for all admits</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>Full tuition waiver + stipend AUD 35,000-45,000/yr, up to 4.5 years (+1 optional fellowship year), plus substantial research/conference travel funding.</t>
+          <t>All successful full-time PhD admits receive a teaching/research assistantship with a monthly stipend of ~HK$19,100. HKPFS awardees additionally receive a full tuition waiver plus HK$40,000 (year 1) / HK$20,000/year (subsequent years) and housing benefits. Local students separately receive a government tuition waiver. Cross-reference the cross-institution HKPFS scheme already tracked (ASA-03).</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>Confirmed EOI window remains closed with no new window announced; added program structure and English-test details</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>Seed entry Aug 2026 — EOI window closed 15 Aug 2026, still no next window announced as of this update</t>
+          <t>New find Aug 2026; distinct from HKU (ASA-08) and the cross-institution HKPFS scheme (ASA-03) — CUHK guarantees baseline assistantship funding to all admits independent of HKPFS.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>AUS-01</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>PhD</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>PhD in Economics</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Australian National University (ANU)</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>#124</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Canberra</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>https://cbe.anu.edu.au/study/graduate-research-programs/doctor-philosophy-phd/phd-economics</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>6.5 overall (no band below 6.0)</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>570 (paper-based; essay ≥4.5)</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Mandatory (code 7833); exempt if ANU Econ Honours/Masters</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Pre-PhD summer course required, Jan-Feb, arriving 4-6 weeks before semester</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>February (Semester 1); Semester 2 entry possible (July)</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>For Feb 2027 start: international scholarship applicants before 31 Aug 2026 (imminent — 2 days away as of 29 Aug 2026, reconfirmed still live via search corroboration of the official ANU text), standard before 31 Oct 2026; Sem 2 entry before 31 Mar</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>urgent</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>Australian Government RTP Stipend: AUD $39,069/year (2026 full-time base rate, ANU-wide), paid fortnightly, up to 3.5 years. Some HDR supplementary scholarships add AUD $7,000/year on top, for up to 3 years. Domestic candidates pay no tuition (RTP-covered); international candidates can compete for HDR Fee Remission Merit Scholarships covering up to 4 years.</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>Reconfirmed the imminent 31 Aug 2026 deadline is still live (ANU site returned HTTP 504 to direct fetch this pass, confirmed instead via search corroboration of the official text); set 7-day reminder flag</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>Seed entry Aug 2026 — international scholarship deadline is imminent (2 days away as of this update)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>AUS-02</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>PhD</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Doctoral Program in Economics</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>University of Melbourne</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>#151</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>https://study.unimelb.edu.au/find/courses/graduate/doctoral-program-in-economics/how-to-apply/</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>7.0 overall (7.0 writing, no band below 6.0)</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>94 iBT (W27/S18/R13/L13)</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Not mentioned in entry requirements</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>PTE Academic 72+ (written 75+); CAE 185+ also accepted; 5-year program (2 coursework + 3 research)</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>March intake</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>March 2027 intake deadline reported as 30 November 2026 — found via search summary only; the official how-to-apply/key-dates pages returned HTTP 403 on every direct fetch attempt this pass, so this date is unconfirmed by primary source and should be manually verified</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>soon</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Not mentioned</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Not detailed — full tuition fee waiver reported (see funding)</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Australian Government Research Training Program (RTP) funded places available: RTP stipend reported at AUD $39,500/year (2026 rate) plus full tuition fee waiver and AUD $15,000 research/conference travel funding for confirmed PhD candidates (unconfirmed by primary source — see deadline note). Program structure: 2-year Master of Commerce coursework + 3-year PhD.</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>Found a reported deadline and funding figures via search, but could not confirm via direct page fetch (403 blocked) — flagged as lower confidence</t>
+        </is>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>Seed entry Aug 2026; unimelb.edu.au pages returned HTTP 403 to automated fetches this pass — recommend a manual browser check before relying on the reported 30 Nov 2026 deadline</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>AUS-03</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>PhD</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>PhD (Economics)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Monash Business School</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>#46</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Melbourne (Clayton)</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>https://www.monash.edu/business/research/phd-programs/scholarships-and-fees</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>7.0 minimum reported (third-party source, not confirmed on official Monash page — page returned HTTP 403 to direct fetch)</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>94 minimum reported (same caveat as IELTS — unconfirmed by primary source)</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Not specified on this page</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Multiple named scholarships stack with base RTP/Monash funding</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Not specified on this page</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Two pathways found (via search — official pages returned HTTP 403 to direct fetch, unconfirmed by primary source): Integrated PhD program (Master of Commerce + PhD), Feb/Semester-1 entry — applications open 1 Jul-31 Aug (closing imminently); Jul/Semester-2 entry — applications open 1 Dec-1 Feb. Separately, general Graduate Research Scholarship rounds: international Round 1 closes 31 Mar, Round 3 closes ~31 Jul/31 Aug; domestic Round 2 closes 31 May, Round 4 closes 31 Oct.</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>urgent</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>International ~AUD $38,900/yr, domestic ~AUD $37,100/yr reported (third-party aggregator source, not confirmed by official Monash page)</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>Donald Cochrane Scholarship: AUD 10,000/yr x 3.5yrs (3 awarded/yr). Dean's Excellence Award: up to AUD 5,000/yr top-up (10/yr). Graduate Research Scholarship: AUD 41,000/yr tuition (~12/yr). Plus university-wide Monash Graduate Scholarship / RTP places — general RTP stipend reported at AUD $37,145/yr (2026 rate) plus a $1,500 relocation allowance (not confirmed Economics-specific).</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>Reconfirmed the imminent ~31 Aug 2026 integrated-pathway deadline is still accurate (search-only — monash.edu continues to block all direct fetches with HTTP 403); found a general RTP stipend figure (AUD $37,145/yr); set 7-day reminder flag</t>
+        </is>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>Seed entry Aug 2026; monash.edu has blocked all automated fetches on every pass so far (scholarships-and-fees, apply, and program pages all 403'd) — every figure in this entry is lower-confidence (search snippets/third-party aggregator only) and needs a manual browser check, especially the imminent 31 Aug 2026 integrated-pathway deadline</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>AUS-04</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>PhD</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>PhD in Economics</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>University of Sydney</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>#87</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>https://www.sydney.edu.au/scholarships/</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Not specified at general program level</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Not specified at general program level</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Not mentioned</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Example named scholarship seen (topic-restricted, econ conflict/ag markets) — general program funding likely via RTP. Material finding: Sydney has no dedicated 'PhD in Economics' program page — the Economics coursework handbook explicitly states it "does not include a research component and thus does not provide a pathway to higher degree by research (e.g. PhD) studies." PhD study is pursued via the general Doctor of Philosophy degree with a nominated Economics supervisor/discipline, not a single named landing page.</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Not specified on this page</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>General Research Training Program (RTP) scholarship rounds for 2027 entry (found via search, not a directly-fetched dedicated Economics PhD page): Research Period 1 &amp; 2 — deadline 11 September 2026; Research Period 3 &amp; 4 — deadline 18 December 2026.</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>urgent</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>1 (for named scholarship example; general program may differ)</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>RTP-style stipend scholarships ~AUD 41,753/yr (base AUD 37,207 + top-up), up to 3 years, seen via School of Economics named scholarship. General RTP funding also available for the PhD program broadly.</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>Found general RTP scholarship round deadlines (11 Sep / 18 Dec 2026); confirmed there is no dedicated Sydney 'PhD in Economics' page — entry is via the general PhD degree with an Economics supervisor; set 30-day reminder flag</t>
+        </is>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>Seed entry Aug 2026; needs a general (non-topic-restricted) funding page check; no dedicated Economics-specific PhD admissions page exists at Sydney</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>AUS-05</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>PhD</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>PhD in Economics</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>UNSW Sydney</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>#80</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>https://www.unsw.edu.au/business/study-with-us/postgraduate-research/phd-degrees/doctor-philosophy-phd-economics</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Not listed on this page (exemptions for AU/CA/UK/US/NZ citizens); non-English-speaking-country applicants need IELTS/TOEFL/PTE/Cambridge or the UNSW Global English Course</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Not listed on this page — see IELTS field for alternatives</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Optional but recommended overall; one source indicates GRE may be specifically required for the Economics stream — this conflicts with the general 'optional' language elsewhere and needs manual confirmation</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Alternative English tests: PTE, Cambridge, or UNSW Global English Course. Program begins with a 1-year Master of Pre-Doctoral Business Studies, followed by 3-3.5 years of doctoral research; direct entry to the 3-year PhD is possible for candidates with first-class Honours/Master's plus independent funding (Stream 2).</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Term 1 – February</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Confirmed still closed as of 23 Aug 2026 (verified directly on program page): EOI window opened 20 March 2026, closed 15 August 2026, no newer/next EOI window posted. Note: a separate 26 August 2026 formal-application deadline exists, but it applies only to candidates already invited to apply from the closed EOI round, not to new applicants.</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Not specified</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>Not detailed (fully funded — see funding)</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>Yes — all admitted students</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>Full tuition waiver + stipend AUD 35,000-45,000/yr, up to 4.5 years (+1 optional fellowship year), plus substantial research/conference travel funding.</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>Confirmed EOI window remains closed with no new window announced; added program structure and English-test details</t>
+        </is>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>Seed entry Aug 2026 — EOI window closed 15 Aug 2026, still no next window announced as of this update</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>AUS-06</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>Doctor of Philosophy (Economics)</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>University of Queensland (School of Economics)</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>#71</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="H36" t="inlineStr">
         <is>
           <t>Brisbane</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>https://economics.uq.edu.au/study/phd</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="J36" t="inlineStr">
         <is>
           <t>Academic overall 6.5, with 6.0 minimum in each of reading/writing/speaking/listening</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="K36" t="inlineStr">
         <is>
           <t>Not specified on the economics-specific page (UQ university-wide PhD pages generally accept TOEFL iBT as an alternative to IELTS)</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr">
+      <c r="L36" t="inlineStr">
         <is>
           <t>Not confirmed as required; application package can include GRE/GMAT score sheets, suggesting optional/supplementary rather than mandatory</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="M36" t="inlineStr">
         <is>
           <t>Academic CV, transcripts; MPhil/research master's options also available; can join a funded project with scholarship support as an alternative entry route</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr">
+      <c r="N36" t="inlineStr">
         <is>
           <t>Quarterly intakes (research quarters begin 1 Jan, 1 Apr, 1 Jul, 1 Oct); applications for RHD programs can be submitted any time</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>Rolling application, but scholarship rounds close on fixed dates — 31 August 2026 and 19 October 2026 rounds cited for upcoming 2027 research quarters</t>
-        </is>
-      </c>
-      <c r="P31" t="inlineStr">
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Confirmed via direct fetch of the UQ Graduate Research School Scholarships page (exact quoted text): 'Monday 31 August 2026 – Application closing date' (Domestic Round 1) and 'Monday 19 October 2026 – Application closing date' (International round), for upcoming 2027 research quarters</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
         <is>
           <t>urgent</t>
         </is>
       </c>
-      <c r="Q31" t="inlineStr">
+      <c r="Q36" t="inlineStr">
         <is>
           <t>Minimum 2 referee reports</t>
         </is>
       </c>
-      <c r="R31" t="inlineStr">
+      <c r="R36" t="inlineStr">
         <is>
           <t>Not specified</t>
         </is>
       </c>
-      <c r="S31" t="inlineStr">
+      <c r="S36" t="inlineStr">
         <is>
           <t>Not specified (international RTP scholarship recipients typically get a full tuition fee offset)</t>
         </is>
       </c>
-      <c r="T31" t="inlineStr">
+      <c r="T36" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U31" t="inlineStr">
-        <is>
-          <t>RTP/UQGRSS provides a tax-free living stipend of AUD $37,500/year (2026 rate, indexed annually) plus, for eligible international candidates, a tuition fee offset; no separate application needed beyond the program EOI.</t>
-        </is>
-      </c>
-      <c r="V31" t="inlineStr">
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>RTP/UQGRSS provides a tax-free living stipend of AUD $39,220/year (2026 rate, indexed annually — updated from a previously-recorded AUD $37,500 figure) plus, for eligible international candidates, a tuition fee offset; no separate application needed beyond the program EOI.</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="W31" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
-      </c>
-      <c r="X31" t="inlineStr">
-        <is>
-          <t>Added (new find)</t>
-        </is>
-      </c>
-      <c r="Y31" t="inlineStr">
-        <is>
-          <t>Scholarship is university-wide (RTP/UQGRSS), not economics-specific, but School of Economics PhD candidates are eligible; confirm current-cycle scholarship closing dates on the UQ Scholarships portal since they shift each year. The 31 Aug 2026 round is imminent.</t>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>Confirmed exact 31 Aug 2026 / 19 Oct 2026 scholarship deadlines via direct official fetch; updated stipend to the current AUD $39,220/yr (2026) rate; set 7-day reminder flag</t>
+        </is>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>Scholarship is university-wide (RTP/UQGRSS), not economics-specific, but School of Economics PhD candidates are eligible. The 31 Aug 2026 round is imminent — 2 days away as of this update.</t>
         </is>
       </c>
     </row>
@@ -4503,13 +5138,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -4543,152 +5178,152 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>EUR-01</t>
+          <t>EUR-17</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
+          <t>PhD in Economics — Vienna Graduate School of Economics (VGSE) — University of Vienna / WU Vienna</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Filled in IELTS/TOEFL/GRE, references, tuition and scholarship amounts; flagged a cohort-year labeling ambiguity in the official deadline text.</t>
+          <t>New find: FWF-grant-funded PhD positions at the University of Vienna; admission-round dates inconsistent across sources, recommend a manual spot-check.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>EUR-02</t>
+          <t>EUR-18</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
+          <t>PhD in Economics — Tilburg University (CentER Graduate School)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Found the M2 ETE application window (10-20 Apr, recurring) and language/GRE/fee requirements — PhD entry is via M2 ETE only, not a standalone application.</t>
+          <t>New find: PhD structured as a salaried employment contract (~EUR 2,750-3,500/month); official site blocked automated fetches, several fields search-only.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>EUR-10</t>
+          <t>EUR-19</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
+          <t>Doctoral Programme in Economics — KU Leuven (Faculty of Economics and Business)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Filled in deadline (31 Mar annually), GRE/reference requirements, and ZEW Cooperation Track funding — previously the least-detailed entry in the tracker.</t>
+          <t>New find: RePEc ~#40, funded PhD positions up to 4 years plus IRO Doctoral Scholarships for developing-country students; deadlines are vacancy-by-vacancy.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>EUR-11</t>
+          <t>EUR-20</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>PhD in Economics and Finance — Bocconi University</t>
+          <t>PhD Program (Economics track) — Berlin School of Economics (BSE)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Confirmed the 2026-27 cycle (ordinary + FIS call) is fully closed and the 2027-28 cycle is not yet announced; added test-requirement and fee detail.</t>
+          <t>New find: joint Berlin-area doctoral school, funded via a EUR 1,650/month qualification-phase stipend then dissertation-phase employment.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>ASA-09</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>PhD in Economics — Chinese University of Hong Kong (CUHK), Department of Economics</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Confirmed deadlines unchanged; added admission requirement detail.</t>
+          <t>New find: guaranteed teaching/research assistantship (~HK$19,100/month) for all admits, independent of the HKPFS scheme already tracked (ASA-03).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>ASA-04</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
+          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -4698,14 +5333,14 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr) and fees; upgraded funding_status from Likely to Yes.</t>
+          <t>Confirmed application windows (Aug intake: 1 Oct-15 Nov; Jan intake: 1 Jun-31 Jul), referee/fee requirements, and Graduate Assistantship Programme detail via direct official fetch; urgency upgraded from tba to soon.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -4725,14 +5360,14 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Site unreachable again this pass (DNS failure, confirmed via two methods); flagged an unconfirmed lead on a possible 2023 admission-policy change limiting PhD entry to internal Master's completers.</t>
+          <t>Corroborated via search snippets (site unreachable for a third consecutive pass) that UTIPE has restricted direct external PhD entry since April 2023 to applicants with 2+ years research experience abroad.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4752,14 +5387,14 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Located the correct department admissions page; found intake-cycle pattern, AO exam routes, and precise RePEc rank (#390).</t>
+          <t>Found the Spring-intake AO-exam submission window (~14-17 Oct, recurring annually) and fee figures via search corroboration; urgency upgraded from tba to soon.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -4779,14 +5414,14 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Found university-wide test-score/fee requirements and admission-cycle pattern; department-specific PhD funding still unconfirmed.</t>
+          <t>Confirmed via direct fetch of the department's own PhD page that no department-specific deadlines, fees, or funding statement exist — resolves prior ambiguity; funding runs entirely through university-wide scholarships.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4801,66 +5436,66 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Confirmed the imminent 31 Aug 2026 international scholarship deadline is still live; added RTP stipend figures; set 30-day reminder flag.</t>
+          <t>7-day reminder: the 31 Aug 2026 international scholarship deadline is confirmed still live via search corroboration (ANU site returned HTTP 504 to direct fetch).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics — University of Melbourne</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Found a reported Nov 2026 deadline and RTP stipend figures via search — official pages blocked automated fetches (HTTP 403), so flagged as lower confidence pending manual check.</t>
+          <t>7-day reminder: the imminent ~31 Aug 2026 integrated-pathway deadline is reconfirmed via search (monash.edu still blocking direct fetch); added a general RTP stipend figure (AUD $37,145/yr).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Updated</t>
+          <t>Deadline reminder</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Found an application-window pattern suggesting an imminent (~31 Aug 2026) integrated-pathway deadline; monash.edu blocked all direct fetches (HTTP 403), so figures are lower-confidence; set 30-day reminder flag.</t>
+          <t>7-day reminder: confirmed exact 31 Aug 2026 / 19 Oct 2026 scholarship deadlines via direct official fetch; updated stipend to AUD $39,220/yr (2026 rate).</t>
         </is>
       </c>
     </row>
@@ -4872,12 +5507,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>EUR-01</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -4887,7 +5522,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Found general RTP scholarship deadlines (11 Sep / 18 Dec 2026); confirmed Sydney has no dedicated 'PhD in Economics' page — entry is via the general PhD degree; set 30-day reminder flag.</t>
+          <t>Filled in IELTS/TOEFL/GRE, references, tuition and scholarship amounts; flagged a cohort-year labeling ambiguity in the official deadline text.</t>
         </is>
       </c>
     </row>
@@ -4899,12 +5534,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>AUS-05</t>
+          <t>EUR-02</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>PhD in Economics — UNSW Sydney</t>
+          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -4914,7 +5549,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Confirmed the EOI window remains closed with no new window announced; added program-structure and English-test detail.</t>
+          <t>Found the M2 ETE application window (10-20 Apr, recurring) and language/GRE/fee requirements — PhD entry is via M2 ETE only, not a standalone application.</t>
         </is>
       </c>
     </row>
@@ -4926,22 +5561,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>EUR-13</t>
+          <t>EUR-10</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MRes/PhD in Economics — London School of Economics (LSE)</t>
+          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>New find: RePEc #16, funded via LSE PhD Studentships and ESRC studentships.</t>
+          <t>Filled in deadline (31 Mar annually), GRE/reference requirements, and ZEW Cooperation Track funding — previously the least-detailed entry in the tracker.</t>
         </is>
       </c>
     </row>
@@ -4953,22 +5588,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>EUR-14</t>
+          <t>EUR-11</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MRes/PhD in Finance &amp; Economics — University of Warwick (Warwick Business School)</t>
+          <t>PhD in Economics and Finance — Bocconi University</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>New find: RePEc #37, fully funded (fee waiver + stipend) for all successful applicants.</t>
+          <t>Confirmed the 2026-27 cycle (ordinary + FIS call) is fully closed and the 2027-28 cycle is not yet announced; added test-requirement and fee detail.</t>
         </is>
       </c>
     </row>
@@ -4980,22 +5615,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>EUR-15</t>
+          <t>ASA-01</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>PhD in Economics (Zurich Graduate School of Economics) — University of Zurich</t>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>New find: RePEc #32, departmental scholarships from year 1 plus a competitive UBS Center Scholarship.</t>
+          <t>Confirmed deadlines unchanged; added admission requirement detail.</t>
         </is>
       </c>
     </row>
@@ -5007,22 +5642,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>EUR-16</t>
+          <t>ASA-02</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>PhD Programme in Economics — University of Copenhagen (Department of Economics)</t>
+          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>New find: RePEc #54, salaried PhD position under the Danish state academic-union pay scale (~EUR 4,150/month).</t>
+          <t>Found explicit departmental Postgraduate Studentship funding (HK$229,620/yr) and fees; upgraded funding_status from Likely to Yes.</t>
         </is>
       </c>
     </row>
@@ -5034,22 +5669,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ASA-08</t>
+          <t>ASA-05</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>PhD in Business (Economics track) — University of Hong Kong (Faculty of Business and Economics)</t>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>New find: RePEc #106, guaranteed Postgraduate Scholarship funding (HK$19,135+/month) independent of the HKPFS scheme already tracked.</t>
+          <t>Site unreachable again this pass (DNS failure, confirmed via two methods); flagged an unconfirmed lead on a possible 2023 admission-policy change limiting PhD entry to internal Master's completers.</t>
         </is>
       </c>
     </row>
@@ -5061,346 +5696,346 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>AUS-06</t>
+          <t>ASA-06</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Added (new find)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>New find: RePEc #71, RTP/UQGRSS stipend AUD $37,500/yr; flagged an imminent 31 Aug 2026 scholarship round.</t>
+          <t>Located the correct department admissions page; found intake-cycle pattern, AO exam routes, and precise RePEc rank (#390).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>EUR-01</t>
+          <t>ASA-07</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Found university-wide test-score/fee requirements and admission-cycle pattern; department-specific PhD funding still unconfirmed.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>EUR-02</t>
+          <t>AUS-01</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
+          <t>PhD in Economics — Australian National University (ANU)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Confirmed the imminent 31 Aug 2026 international scholarship deadline is still live; added RTP stipend figures; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>EUR-03</t>
+          <t>AUS-02</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
+          <t>Doctoral Program in Economics — University of Melbourne</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Found a reported Nov 2026 deadline and RTP stipend figures via search — official pages blocked automated fetches (HTTP 403), so flagged as lower confidence pending manual check.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>EUR-04</t>
+          <t>AUS-03</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Combined M.Sc. Economic Research / Doctoral Program — Bonn Graduate School of Economics (BGSE)</t>
+          <t>PhD (Economics) — Monash Business School</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Found an application-window pattern suggesting an imminent (~31 Aug 2026) integrated-pathway deadline; monash.edu blocked all direct fetches (HTTP 403), so figures are lower-confidence; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>EUR-05</t>
+          <t>AUS-04</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>PhD in Economics — CEMFI</t>
+          <t>PhD in Economics — University of Sydney</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Found general RTP scholarship deadlines (11 Sep / 18 Dec 2026); confirmed Sydney has no dedicated 'PhD in Economics' page — entry is via the general PhD degree; set 30-day reminder flag.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>EUR-06</t>
+          <t>AUS-05</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Master's in Economics — Barcelona School of Economics (BSE)</t>
+          <t>PhD in Economics — UNSW Sydney</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>Confirmed the EOI window remains closed with no new window announced; added program-structure and English-test detail.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>EUR-07</t>
+          <t>EUR-13</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PhD Program — Paris School of Economics (PSE)</t>
+          <t>MRes/PhD in Economics — London School of Economics (LSE)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #16, funded via LSE PhD Studentships and ESRC studentships.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>EUR-08</t>
+          <t>EUR-14</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PhD Programme in Economics — Stockholm University / IIES</t>
+          <t>MRes/PhD in Finance &amp; Economics — University of Warwick (Warwick Business School)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #37, fully funded (fee waiver + stipend) for all successful applicants.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>EUR-09</t>
+          <t>EUR-15</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MPhil + DPhil in Economics — University of Oxford</t>
+          <t>PhD in Economics (Zurich Graduate School of Economics) — University of Zurich</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #32, departmental scholarships from year 1 plus a competitive UBS Center Scholarship.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>EUR-10</t>
+          <t>EUR-16</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
+          <t>PhD Programme in Economics — University of Copenhagen (Department of Economics)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #54, salaried PhD position under the Danish state academic-union pay scale (~EUR 4,150/month).</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>EUR-11</t>
+          <t>ASA-08</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>PhD in Economics and Finance — Bocconi University</t>
+          <t>PhD in Business (Economics track) — University of Hong Kong (Faculty of Business and Economics)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #106, guaranteed Postgraduate Scholarship funding (HK$19,135+/month) independent of the HKPFS scheme already tracked.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>EUR-12</t>
+          <t>AUS-06</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
+          <t>Doctor of Philosophy (Economics) — University of Queensland (School of Economics)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Added (seed)</t>
+          <t>Added (new find)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Initial research pass — program added to tracker.</t>
+          <t>New find: RePEc #71, RTP/UQGRSS stipend AUD $37,500/yr; flagged an imminent 31 Aug 2026 scholarship round.</t>
         </is>
       </c>
     </row>
@@ -5412,12 +6047,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ASA-01</t>
+          <t>EUR-01</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>PhD in Economics — National University of Singapore (NUS)</t>
+          <t>Research Master in Economics — Tinbergen Institute (UvA / VU / Erasmus)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -5439,12 +6074,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ASA-02</t>
+          <t>EUR-02</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
+          <t>Doctoral Program — Toulouse School of Economics (TSE)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -5466,12 +6101,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ASA-03</t>
+          <t>EUR-03</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Hong Kong PhD Fellowship Scheme (HKPFS) — Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
+          <t>Doctoral Programme in Economics — European University Institute (EUI)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -5493,12 +6128,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ASA-04</t>
+          <t>EUR-04</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
+          <t>Combined M.Sc. Economic Research / Doctoral Program — Bonn Graduate School of Economics (BGSE)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -5520,12 +6155,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ASA-05</t>
+          <t>EUR-05</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>International Program in Economics (PhD) — University of Tokyo</t>
+          <t>PhD in Economics — CEMFI</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -5547,12 +6182,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ASA-06</t>
+          <t>EUR-06</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+          <t>Master's in Economics — Barcelona School of Economics (BSE)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -5574,12 +6209,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ASA-07</t>
+          <t>EUR-07</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+          <t>PhD Program — Paris School of Economics (PSE)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -5601,12 +6236,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>AUS-01</t>
+          <t>EUR-08</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>PhD in Economics — Australian National University (ANU)</t>
+          <t>PhD Programme in Economics — Stockholm University / IIES</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -5628,12 +6263,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>AUS-02</t>
+          <t>EUR-09</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Doctoral Program in Economics — University of Melbourne</t>
+          <t>MPhil + DPhil in Economics — University of Oxford</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -5655,12 +6290,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>AUS-03</t>
+          <t>EUR-10</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>PhD (Economics) — Monash Business School</t>
+          <t>CDSE Doctoral Program in Economics — University of Mannheim (CDSE)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -5682,12 +6317,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>AUS-04</t>
+          <t>EUR-11</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>PhD in Economics — University of Sydney</t>
+          <t>PhD in Economics and Finance — Bocconi University</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -5709,20 +6344,344 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
+          <t>EUR-12</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Economics MRes + MPhil/PhD — University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ASA-01</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>PhD in Economics — National University of Singapore (NUS)</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>ASA-02</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>MPhil/PhD in Economics — Hong Kong University of Science and Technology (HKUST)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>ASA-03</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Hong Kong PhD Fellowship Scheme (HKPFS) — Hong Kong universities incl. CUHK / HKUST / HKU / CityU (Economics eligible)</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>ASA-04</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>PhD in Economics — Nanyang Technological University (NTU Singapore)</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>ASA-05</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>International Program in Economics (PhD) — University of Tokyo</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>ASA-06</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Graduate School of Economics (PhD) — Hitotsubashi University</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>ASA-07</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Department of Economics (PhD) — Seoul National University (SNU)</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>AUS-01</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>PhD in Economics — Australian National University (ANU)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>AUS-02</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Doctoral Program in Economics — University of Melbourne</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>AUS-03</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>PhD (Economics) — Monash Business School</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>AUS-04</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>PhD in Economics — University of Sydney</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Added (seed)</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Initial research pass — program added to tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
           <t>AUS-05</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>PhD in Economics — UNSW Sydney</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D57" t="inlineStr">
         <is>
           <t>Added (seed)</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E57" t="inlineStr">
         <is>
           <t>Initial research pass — program added to tracker.</t>
         </is>

</xml_diff>